<commit_message>
add codex harness and lab validation improvements
</commit_message>
<xml_diff>
--- a/진단항목통합.xlsx
+++ b/진단항목통합.xlsx
@@ -1054,7 +1054,7 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>CLD-KVM-01</t>
+          <t>CSAP-KVM-01</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>CLD-KVM-02</t>
+          <t>CSAP-KVM-02</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
@@ -1164,7 +1164,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>CLD-KVM-03</t>
+          <t>CSAP-KVM-03</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>CLD-KVM-04</t>
+          <t>CSAP-KVM-04</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>CLD-KVM-05</t>
+          <t>CSAP-KVM-05</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>CLD-KVM-06</t>
+          <t>CSAP-KVM-06</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>HV-01</t>
+          <t>ISMS-HV-01</t>
         </is>
       </c>
       <c r="E9" s="8" t="inlineStr">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>HV-02</t>
+          <t>ISMS-HV-02</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -1565,7 +1565,7 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>HV-04</t>
+          <t>ISMS-HV-04</t>
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr">
@@ -1632,7 +1632,7 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>HV-05</t>
+          <t>ISMS-HV-05</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -1699,7 +1699,7 @@
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>HV-06</t>
+          <t>ISMS-HV-06</t>
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>HV-07</t>
+          <t>ISMS-HV-07</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>HV-08</t>
+          <t>ISMS-HV-08</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>HV-10</t>
+          <t>ISMS-HV-10</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -1989,7 +1989,7 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>HV-14</t>
+          <t>ISMS-HV-14</t>
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>HV-15</t>
+          <t>ISMS-HV-15</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-02 / HV-04</t>
+          <t>CSAP-Xenserver-02 / ISMS-HV-04</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-01</t>
+          <t>CSAP-Xenserver-01</t>
         </is>
       </c>
       <c r="E21" s="8" t="inlineStr">
@@ -2299,7 +2299,7 @@
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-03</t>
+          <t>CSAP-Xenserver-03</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-04</t>
+          <t>CSAP-Xenserver-04</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-05</t>
+          <t>CSAP-Xenserver-05</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
@@ -2457,7 +2457,7 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-06</t>
+          <t>CSAP-Xenserver-06</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-07</t>
+          <t>CSAP-Xenserver-07</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -2575,7 +2575,7 @@
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-08</t>
+          <t>CSAP-Xenserver-08</t>
         </is>
       </c>
       <c r="E27" s="8" t="inlineStr">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-09</t>
+          <t>CSAP-Xenserver-09</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-10</t>
+          <t>CSAP-Xenserver-10</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
@@ -2755,7 +2755,7 @@
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-11</t>
+          <t>CSAP-Xenserver-11</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-12</t>
+          <t>CSAP-Xenserver-12</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -2881,7 +2881,7 @@
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-13</t>
+          <t>CSAP-Xenserver-13</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-14</t>
+          <t>CSAP-Xenserver-14</t>
         </is>
       </c>
       <c r="E33" s="8" t="inlineStr">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-15</t>
+          <t>CSAP-Xenserver-15</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
@@ -3046,7 +3046,7 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-16</t>
+          <t>CSAP-Xenserver-16</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
@@ -3110,7 +3110,7 @@
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-17</t>
+          <t>CSAP-Xenserver-17</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-18</t>
+          <t>CSAP-Xenserver-18</t>
         </is>
       </c>
       <c r="E37" s="8" t="inlineStr">
@@ -3215,7 +3215,7 @@
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-19</t>
+          <t>CSAP-Xenserver-19</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
@@ -3283,7 +3283,7 @@
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-20</t>
+          <t>CSAP-Xenserver-20</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
@@ -3351,7 +3351,7 @@
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-21</t>
+          <t>CSAP-Xenserver-21</t>
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-22</t>
+          <t>CSAP-Xenserver-22</t>
         </is>
       </c>
       <c r="E41" s="8" t="inlineStr">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-23</t>
+          <t>CSAP-Xenserver-23</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
@@ -3530,7 +3530,7 @@
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-24</t>
+          <t>CSAP-Xenserver-24</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
@@ -3638,7 +3638,7 @@
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-25</t>
+          <t>CSAP-Xenserver-25</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
@@ -3694,7 +3694,7 @@
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-26</t>
+          <t>CSAP-Xenserver-26</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
@@ -3753,7 +3753,7 @@
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-27</t>
+          <t>CSAP-Xenserver-27</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
@@ -3816,7 +3816,7 @@
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-28</t>
+          <t>CSAP-Xenserver-28</t>
         </is>
       </c>
       <c r="E47" s="8" t="inlineStr">
@@ -3874,7 +3874,7 @@
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-29</t>
+          <t>CSAP-Xenserver-29</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
@@ -4015,7 +4015,7 @@
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-30</t>
+          <t>CSAP-Xenserver-30</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
@@ -4079,7 +4079,7 @@
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-31</t>
+          <t>CSAP-Xenserver-31</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
@@ -4155,7 +4155,7 @@
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-32</t>
+          <t>CSAP-Xenserver-32</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>CLD-Xenserver-33</t>
+          <t>CSAP-Xenserver-33</t>
         </is>
       </c>
       <c r="E52" s="8" t="inlineStr">
@@ -4287,7 +4287,7 @@
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>HV-01</t>
+          <t>ISMS-HV-01</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -4360,7 +4360,7 @@
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>HV-02</t>
+          <t>ISMS-HV-02</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
@@ -4464,7 +4464,7 @@
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>HV-05</t>
+          <t>ISMS-HV-05</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
@@ -4563,7 +4563,7 @@
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>HV-06</t>
+          <t>ISMS-HV-06</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
@@ -4636,7 +4636,7 @@
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>HV-08</t>
+          <t>ISMS-HV-08</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
@@ -4707,7 +4707,7 @@
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>HV-10</t>
+          <t>ISMS-HV-10</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
@@ -4770,7 +4770,7 @@
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>HV-14</t>
+          <t>ISMS-HV-14</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
@@ -4833,7 +4833,7 @@
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>HV-19</t>
+          <t>ISMS-HV-19</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr">
@@ -4928,7 +4928,7 @@
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>HV-23</t>
+          <t>ISMS-HV-23</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
@@ -5018,7 +5018,7 @@
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-03 / HV-07</t>
+          <t>CSAP-ESXi-03 / ISMS-HV-07</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
@@ -5145,7 +5145,7 @@
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-05 / HV-12</t>
+          <t>CSAP-ESXi-05 / ISMS-HV-12</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-06 / HV-13</t>
+          <t>CSAP-ESXi-06 / ISMS-HV-13</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
@@ -5329,7 +5329,7 @@
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-08 / HV-22</t>
+          <t>CSAP-ESXi-08 / ISMS-HV-22</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
@@ -5418,7 +5418,7 @@
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-09 / HV-23</t>
+          <t>CSAP-ESXi-09 / ISMS-HV-23</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
@@ -5509,7 +5509,7 @@
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-10 / HV-24</t>
+          <t>CSAP-ESXi-10 / ISMS-HV-24</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr">
@@ -5600,7 +5600,7 @@
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-13 / HV-10</t>
+          <t>CSAP-ESXi-13 / ISMS-HV-10</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
@@ -5698,7 +5698,7 @@
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-21 / HV-11</t>
+          <t>CSAP-ESXi-21 / ISMS-HV-11</t>
         </is>
       </c>
       <c r="E70" s="8" t="inlineStr">
@@ -5796,7 +5796,7 @@
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-01</t>
+          <t>CSAP-ESXi-01</t>
         </is>
       </c>
       <c r="E71" s="8" t="inlineStr">
@@ -5849,7 +5849,7 @@
       </c>
       <c r="D72" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-02</t>
+          <t>CSAP-ESXi-02</t>
         </is>
       </c>
       <c r="E72" s="8" t="inlineStr">
@@ -5931,7 +5931,7 @@
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-04</t>
+          <t>CSAP-ESXi-04</t>
         </is>
       </c>
       <c r="E73" s="8" t="inlineStr">
@@ -5990,7 +5990,7 @@
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-07</t>
+          <t>CSAP-ESXi-07</t>
         </is>
       </c>
       <c r="E74" s="8" t="inlineStr">
@@ -6054,7 +6054,7 @@
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-11</t>
+          <t>CSAP-ESXi-11</t>
         </is>
       </c>
       <c r="E75" s="8" t="inlineStr">
@@ -6110,7 +6110,7 @@
       </c>
       <c r="D76" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-12</t>
+          <t>CSAP-ESXi-12</t>
         </is>
       </c>
       <c r="E76" s="8" t="inlineStr">
@@ -6166,7 +6166,7 @@
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-14</t>
+          <t>CSAP-ESXi-14</t>
         </is>
       </c>
       <c r="E77" s="8" t="inlineStr">
@@ -6230,7 +6230,7 @@
       </c>
       <c r="D78" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-15</t>
+          <t>CSAP-ESXi-15</t>
         </is>
       </c>
       <c r="E78" s="8" t="inlineStr">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-16</t>
+          <t>CSAP-ESXi-16</t>
         </is>
       </c>
       <c r="E79" s="8" t="inlineStr">
@@ -6333,7 +6333,7 @@
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-17</t>
+          <t>CSAP-ESXi-17</t>
         </is>
       </c>
       <c r="E80" s="8" t="inlineStr">
@@ -6386,7 +6386,7 @@
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-18</t>
+          <t>CSAP-ESXi-18</t>
         </is>
       </c>
       <c r="E81" s="8" t="inlineStr">
@@ -6445,7 +6445,7 @@
       </c>
       <c r="D82" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-19</t>
+          <t>CSAP-ESXi-19</t>
         </is>
       </c>
       <c r="E82" s="8" t="inlineStr">
@@ -6507,7 +6507,7 @@
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-20</t>
+          <t>CSAP-ESXi-20</t>
         </is>
       </c>
       <c r="E83" s="8" t="inlineStr">
@@ -6571,7 +6571,7 @@
       </c>
       <c r="D84" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-22</t>
+          <t>CSAP-ESXi-22</t>
         </is>
       </c>
       <c r="E84" s="8" t="inlineStr">
@@ -6632,7 +6632,7 @@
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-23</t>
+          <t>CSAP-ESXi-23</t>
         </is>
       </c>
       <c r="E85" s="8" t="inlineStr">
@@ -6691,7 +6691,7 @@
       </c>
       <c r="D86" s="6" t="inlineStr">
         <is>
-          <t>CLD-ESXi-24</t>
+          <t>CSAP-ESXi-24</t>
         </is>
       </c>
       <c r="E86" s="8" t="inlineStr">
@@ -6744,7 +6744,7 @@
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>HV-01</t>
+          <t>ISMS-HV-01</t>
         </is>
       </c>
       <c r="E87" s="8" t="inlineStr">
@@ -6815,7 +6815,7 @@
       </c>
       <c r="D88" s="6" t="inlineStr">
         <is>
-          <t>HV-02</t>
+          <t>ISMS-HV-02</t>
         </is>
       </c>
       <c r="E88" s="8" t="inlineStr">
@@ -6891,7 +6891,7 @@
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>HV-03</t>
+          <t>ISMS-HV-03</t>
         </is>
       </c>
       <c r="E89" s="8" t="inlineStr">
@@ -6974,7 +6974,7 @@
       </c>
       <c r="D90" s="6" t="inlineStr">
         <is>
-          <t>HV-04</t>
+          <t>ISMS-HV-04</t>
         </is>
       </c>
       <c r="E90" s="8" t="inlineStr">
@@ -7041,7 +7041,7 @@
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>HV-05</t>
+          <t>ISMS-HV-05</t>
         </is>
       </c>
       <c r="E91" s="8" t="inlineStr">
@@ -7112,7 +7112,7 @@
       </c>
       <c r="D92" s="6" t="inlineStr">
         <is>
-          <t>HV-06</t>
+          <t>ISMS-HV-06</t>
         </is>
       </c>
       <c r="E92" s="8" t="inlineStr">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>HV-08</t>
+          <t>ISMS-HV-08</t>
         </is>
       </c>
       <c r="E93" s="8" t="inlineStr">
@@ -7338,7 +7338,7 @@
       </c>
       <c r="D94" s="6" t="inlineStr">
         <is>
-          <t>HV-14</t>
+          <t>ISMS-HV-14</t>
         </is>
       </c>
       <c r="E94" s="8" t="inlineStr">
@@ -7443,7 +7443,7 @@
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>HV-15</t>
+          <t>ISMS-HV-15</t>
         </is>
       </c>
       <c r="E95" s="8" t="inlineStr">
@@ -7566,7 +7566,7 @@
       </c>
       <c r="D96" s="6" t="inlineStr">
         <is>
-          <t>HV-16</t>
+          <t>ISMS-HV-16</t>
         </is>
       </c>
       <c r="E96" s="8" t="inlineStr">
@@ -7633,7 +7633,7 @@
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>HV-17</t>
+          <t>ISMS-HV-17</t>
         </is>
       </c>
       <c r="E97" s="8" t="inlineStr">
@@ -7710,7 +7710,7 @@
       </c>
       <c r="D98" s="6" t="inlineStr">
         <is>
-          <t>HV-18</t>
+          <t>ISMS-HV-18</t>
         </is>
       </c>
       <c r="E98" s="8" t="inlineStr">
@@ -7779,7 +7779,7 @@
       </c>
       <c r="D99" s="6" t="inlineStr">
         <is>
-          <t>HV-19</t>
+          <t>ISMS-HV-19</t>
         </is>
       </c>
       <c r="E99" s="8" t="inlineStr">
@@ -7846,7 +7846,7 @@
       </c>
       <c r="D100" s="6" t="inlineStr">
         <is>
-          <t>HV-20</t>
+          <t>ISMS-HV-20</t>
         </is>
       </c>
       <c r="E100" s="8" t="inlineStr">
@@ -7919,7 +7919,7 @@
       </c>
       <c r="D101" s="6" t="inlineStr">
         <is>
-          <t>HV-21</t>
+          <t>ISMS-HV-21</t>
         </is>
       </c>
       <c r="E101" s="8" t="inlineStr">
@@ -8003,7 +8003,7 @@
       </c>
       <c r="D103" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-01 / U-01</t>
+          <t>CSAP-Linux-01 / ISMS-U-01</t>
         </is>
       </c>
       <c r="E103" s="8" t="inlineStr">
@@ -8118,7 +8118,7 @@
       </c>
       <c r="D104" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-03 / U-03</t>
+          <t>CSAP-Linux-03 / ISMS-U-03</t>
         </is>
       </c>
       <c r="E104" s="8" t="inlineStr">
@@ -8290,7 +8290,7 @@
       </c>
       <c r="D105" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-05 / U-04</t>
+          <t>CSAP-Linux-05 / ISMS-U-04</t>
         </is>
       </c>
       <c r="E105" s="8" t="inlineStr">
@@ -8372,7 +8372,7 @@
       </c>
       <c r="D106" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-06 / U-14</t>
+          <t>CSAP-Linux-06 / ISMS-U-14</t>
         </is>
       </c>
       <c r="E106" s="8" t="inlineStr">
@@ -8474,7 +8474,7 @@
       </c>
       <c r="D107" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-07 / U-15</t>
+          <t>CSAP-Linux-07 / ISMS-U-15</t>
         </is>
       </c>
       <c r="E107" s="8" t="inlineStr">
@@ -8567,7 +8567,7 @@
       </c>
       <c r="D108" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-08 / U-16</t>
+          <t>CSAP-Linux-08 / ISMS-U-16</t>
         </is>
       </c>
       <c r="E108" s="8" t="inlineStr">
@@ -8647,7 +8647,7 @@
       </c>
       <c r="D109" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-09 / U-18</t>
+          <t>CSAP-Linux-09 / ISMS-U-18</t>
         </is>
       </c>
       <c r="E109" s="8" t="inlineStr">
@@ -8721,7 +8721,7 @@
       </c>
       <c r="D110" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-10 / U-19</t>
+          <t>CSAP-Linux-10 / ISMS-U-19</t>
         </is>
       </c>
       <c r="E110" s="8" t="inlineStr">
@@ -8797,7 +8797,7 @@
       </c>
       <c r="D111" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-11 / U-20</t>
+          <t>CSAP-Linux-11 / ISMS-U-20</t>
         </is>
       </c>
       <c r="E111" s="8" t="inlineStr">
@@ -8906,7 +8906,7 @@
       </c>
       <c r="D112" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-12 / U-21</t>
+          <t>CSAP-Linux-12 / ISMS-U-21</t>
         </is>
       </c>
       <c r="E112" s="8" t="inlineStr">
@@ -8988,7 +8988,7 @@
       </c>
       <c r="D113" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-13 / U-22</t>
+          <t>CSAP-Linux-13 / ISMS-U-22</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
@@ -9064,7 +9064,7 @@
       </c>
       <c r="D114" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-14 / U-23</t>
+          <t>CSAP-Linux-14 / ISMS-U-23</t>
         </is>
       </c>
       <c r="E114" s="8" t="inlineStr">
@@ -9159,7 +9159,7 @@
       </c>
       <c r="D115" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-15 / U-24</t>
+          <t>CSAP-Linux-15 / ISMS-U-24</t>
         </is>
       </c>
       <c r="E115" s="8" t="inlineStr">
@@ -9249,7 +9249,7 @@
       </c>
       <c r="D116" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-16 / U-25</t>
+          <t>CSAP-Linux-16 / ISMS-U-25</t>
         </is>
       </c>
       <c r="E116" s="8" t="inlineStr">
@@ -9337,7 +9337,7 @@
       </c>
       <c r="D117" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-17 / U-27</t>
+          <t>CSAP-Linux-17 / ISMS-U-27</t>
         </is>
       </c>
       <c r="E117" s="8" t="inlineStr">
@@ -9461,7 +9461,7 @@
       </c>
       <c r="D118" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-18 / U-28</t>
+          <t>CSAP-Linux-18 / ISMS-U-28</t>
         </is>
       </c>
       <c r="E118" s="8" t="inlineStr">
@@ -9611,7 +9611,7 @@
       </c>
       <c r="D119" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-19 / U-29</t>
+          <t>CSAP-Linux-19 / ISMS-U-29</t>
         </is>
       </c>
       <c r="E119" s="8" t="inlineStr">
@@ -9695,7 +9695,7 @@
       </c>
       <c r="D120" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-20 / U-34</t>
+          <t>CSAP-Linux-20 / ISMS-U-34</t>
         </is>
       </c>
       <c r="E120" s="8" t="inlineStr">
@@ -9783,7 +9783,7 @@
       </c>
       <c r="D121" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-22 / U-36</t>
+          <t>CSAP-Linux-22 / ISMS-U-36</t>
         </is>
       </c>
       <c r="E121" s="8" t="inlineStr">
@@ -9910,7 +9910,7 @@
       </c>
       <c r="D122" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-23 / U-38</t>
+          <t>CSAP-Linux-23 / ISMS-U-38</t>
         </is>
       </c>
       <c r="E122" s="8" t="inlineStr">
@@ -10054,7 +10054,7 @@
       </c>
       <c r="D123" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-24 / U-39</t>
+          <t>CSAP-Linux-24 / ISMS-U-39</t>
         </is>
       </c>
       <c r="E123" s="8" t="inlineStr">
@@ -10138,7 +10138,7 @@
       </c>
       <c r="D124" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-25 / U-40</t>
+          <t>CSAP-Linux-25 / ISMS-U-40</t>
         </is>
       </c>
       <c r="E124" s="8" t="inlineStr">
@@ -10241,7 +10241,7 @@
       </c>
       <c r="D125" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-26 / U-41</t>
+          <t>CSAP-Linux-26 / ISMS-U-41</t>
         </is>
       </c>
       <c r="E125" s="8" t="inlineStr">
@@ -10333,7 +10333,7 @@
       </c>
       <c r="D126" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-27 / U-42</t>
+          <t>CSAP-Linux-27 / ISMS-U-42</t>
         </is>
       </c>
       <c r="E126" s="8" t="inlineStr">
@@ -10457,7 +10457,7 @@
       </c>
       <c r="D127" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-28 / U-43</t>
+          <t>CSAP-Linux-28 / ISMS-U-43</t>
         </is>
       </c>
       <c r="E127" s="8" t="inlineStr">
@@ -10536,7 +10536,7 @@
       </c>
       <c r="D128" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-29 / U-44</t>
+          <t>CSAP-Linux-29 / ISMS-U-44</t>
         </is>
       </c>
       <c r="E128" s="8" t="inlineStr">
@@ -10664,7 +10664,7 @@
       </c>
       <c r="D129" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-30 / U-45</t>
+          <t>CSAP-Linux-30 / ISMS-U-45</t>
         </is>
       </c>
       <c r="E129" s="8" t="inlineStr">
@@ -10813,7 +10813,7 @@
       </c>
       <c r="D130" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-31 / U-47</t>
+          <t>CSAP-Linux-31 / ISMS-U-47</t>
         </is>
       </c>
       <c r="E130" s="8" t="inlineStr">
@@ -10987,7 +10987,7 @@
       </c>
       <c r="D131" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-32 / U-46</t>
+          <t>CSAP-Linux-32 / ISMS-U-46</t>
         </is>
       </c>
       <c r="E131" s="8" t="inlineStr">
@@ -11102,7 +11102,7 @@
       </c>
       <c r="D132" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-33 / U-49</t>
+          <t>CSAP-Linux-33 / ISMS-U-49</t>
         </is>
       </c>
       <c r="E132" s="8" t="inlineStr">
@@ -11196,7 +11196,7 @@
       </c>
       <c r="D133" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-34 / U-50</t>
+          <t>CSAP-Linux-34 / ISMS-U-50</t>
         </is>
       </c>
       <c r="E133" s="8" t="inlineStr">
@@ -11300,7 +11300,7 @@
       </c>
       <c r="D134" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-35 / U-64</t>
+          <t>CSAP-Linux-35 / ISMS-U-64</t>
         </is>
       </c>
       <c r="E134" s="8" t="inlineStr">
@@ -11386,7 +11386,7 @@
       </c>
       <c r="D135" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-02</t>
+          <t>CSAP-Linux-02</t>
         </is>
       </c>
       <c r="E135" s="8" t="inlineStr">
@@ -11460,7 +11460,7 @@
       </c>
       <c r="D136" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-04</t>
+          <t>CSAP-Linux-04</t>
         </is>
       </c>
       <c r="E136" s="8" t="inlineStr">
@@ -11516,7 +11516,7 @@
       </c>
       <c r="D137" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-21</t>
+          <t>CSAP-Linux-21</t>
         </is>
       </c>
       <c r="E137" s="8" t="inlineStr">
@@ -11577,7 +11577,7 @@
       </c>
       <c r="D138" s="6" t="inlineStr">
         <is>
-          <t>CLD-Linux-36</t>
+          <t>CSAP-Linux-36</t>
         </is>
       </c>
       <c r="E138" s="8" t="inlineStr">
@@ -11639,7 +11639,7 @@
       </c>
       <c r="D139" s="6" t="inlineStr">
         <is>
-          <t>U-02</t>
+          <t>ISMS-U-02</t>
         </is>
       </c>
       <c r="E139" s="8" t="inlineStr">
@@ -11840,7 +11840,7 @@
       </c>
       <c r="D140" s="6" t="inlineStr">
         <is>
-          <t>U-05</t>
+          <t>ISMS-U-05</t>
         </is>
       </c>
       <c r="E140" s="8" t="inlineStr">
@@ -11911,7 +11911,7 @@
       </c>
       <c r="D141" s="6" t="inlineStr">
         <is>
-          <t>U-06</t>
+          <t>ISMS-U-06</t>
         </is>
       </c>
       <c r="E141" s="8" t="inlineStr">
@@ -12015,7 +12015,7 @@
       </c>
       <c r="D142" s="6" t="inlineStr">
         <is>
-          <t>U-07</t>
+          <t>ISMS-U-07</t>
         </is>
       </c>
       <c r="E142" s="8" t="inlineStr">
@@ -12085,7 +12085,7 @@
       </c>
       <c r="D143" s="6" t="inlineStr">
         <is>
-          <t>U-08</t>
+          <t>ISMS-U-08</t>
         </is>
       </c>
       <c r="E143" s="8" t="inlineStr">
@@ -12150,7 +12150,7 @@
       </c>
       <c r="D144" s="6" t="inlineStr">
         <is>
-          <t>U-09</t>
+          <t>ISMS-U-09</t>
         </is>
       </c>
       <c r="E144" s="8" t="inlineStr">
@@ -12216,7 +12216,7 @@
       </c>
       <c r="D145" s="6" t="inlineStr">
         <is>
-          <t>U-10</t>
+          <t>ISMS-U-10</t>
         </is>
       </c>
       <c r="E145" s="8" t="inlineStr">
@@ -12282,7 +12282,7 @@
       </c>
       <c r="D146" s="6" t="inlineStr">
         <is>
-          <t>U-11</t>
+          <t>ISMS-U-11</t>
         </is>
       </c>
       <c r="E146" s="8" t="inlineStr">
@@ -12353,7 +12353,7 @@
       </c>
       <c r="D147" s="6" t="inlineStr">
         <is>
-          <t>U-12</t>
+          <t>ISMS-U-12</t>
         </is>
       </c>
       <c r="E147" s="8" t="inlineStr">
@@ -12424,7 +12424,7 @@
       </c>
       <c r="D148" s="6" t="inlineStr">
         <is>
-          <t>U-13</t>
+          <t>ISMS-U-13</t>
         </is>
       </c>
       <c r="E148" s="8" t="inlineStr">
@@ -12501,7 +12501,7 @@
       </c>
       <c r="D149" s="6" t="inlineStr">
         <is>
-          <t>U-17</t>
+          <t>ISMS-U-17</t>
         </is>
       </c>
       <c r="E149" s="8" t="inlineStr">
@@ -12580,7 +12580,7 @@
       </c>
       <c r="D150" s="6" t="inlineStr">
         <is>
-          <t>U-26</t>
+          <t>ISMS-U-26</t>
         </is>
       </c>
       <c r="E150" s="8" t="inlineStr">
@@ -12641,7 +12641,7 @@
       </c>
       <c r="D151" s="6" t="inlineStr">
         <is>
-          <t>U-30</t>
+          <t>ISMS-U-30</t>
         </is>
       </c>
       <c r="E151" s="8" t="inlineStr">
@@ -12712,7 +12712,7 @@
       </c>
       <c r="D152" s="6" t="inlineStr">
         <is>
-          <t>U-31</t>
+          <t>ISMS-U-31</t>
         </is>
       </c>
       <c r="E152" s="8" t="inlineStr">
@@ -12783,7 +12783,7 @@
       </c>
       <c r="D153" s="6" t="inlineStr">
         <is>
-          <t>U-32</t>
+          <t>ISMS-U-32</t>
         </is>
       </c>
       <c r="E153" s="8" t="inlineStr">
@@ -12854,7 +12854,7 @@
       </c>
       <c r="D154" s="6" t="inlineStr">
         <is>
-          <t>U-33</t>
+          <t>ISMS-U-33</t>
         </is>
       </c>
       <c r="E154" s="8" t="inlineStr">
@@ -12925,7 +12925,7 @@
       </c>
       <c r="D155" s="6" t="inlineStr">
         <is>
-          <t>U-35</t>
+          <t>ISMS-U-35</t>
         </is>
       </c>
       <c r="E155" s="8" t="inlineStr">
@@ -13068,7 +13068,7 @@
       </c>
       <c r="D156" s="6" t="inlineStr">
         <is>
-          <t>U-37</t>
+          <t>ISMS-U-37</t>
         </is>
       </c>
       <c r="E156" s="8" t="inlineStr">
@@ -13143,7 +13143,7 @@
       </c>
       <c r="D157" s="6" t="inlineStr">
         <is>
-          <t>U-48</t>
+          <t>ISMS-U-48</t>
         </is>
       </c>
       <c r="E157" s="8" t="inlineStr">
@@ -13243,7 +13243,7 @@
       </c>
       <c r="D158" s="6" t="inlineStr">
         <is>
-          <t>U-51</t>
+          <t>ISMS-U-51</t>
         </is>
       </c>
       <c r="E158" s="8" t="inlineStr">
@@ -13328,7 +13328,7 @@
       </c>
       <c r="D159" s="6" t="inlineStr">
         <is>
-          <t>U-52</t>
+          <t>ISMS-U-52</t>
         </is>
       </c>
       <c r="E159" s="8" t="inlineStr">
@@ -13435,7 +13435,7 @@
       </c>
       <c r="D160" s="6" t="inlineStr">
         <is>
-          <t>U-53</t>
+          <t>ISMS-U-53</t>
         </is>
       </c>
       <c r="E160" s="8" t="inlineStr">
@@ -13520,7 +13520,7 @@
       </c>
       <c r="D161" s="6" t="inlineStr">
         <is>
-          <t>U-54</t>
+          <t>ISMS-U-54</t>
         </is>
       </c>
       <c r="E161" s="8" t="inlineStr">
@@ -13629,7 +13629,7 @@
       </c>
       <c r="D162" s="6" t="inlineStr">
         <is>
-          <t>U-55</t>
+          <t>ISMS-U-55</t>
         </is>
       </c>
       <c r="E162" s="8" t="inlineStr">
@@ -13701,7 +13701,7 @@
       </c>
       <c r="D163" s="6" t="inlineStr">
         <is>
-          <t>U-56</t>
+          <t>ISMS-U-56</t>
         </is>
       </c>
       <c r="E163" s="8" t="inlineStr">
@@ -13907,7 +13907,7 @@
       </c>
       <c r="D164" s="6" t="inlineStr">
         <is>
-          <t>U-57</t>
+          <t>ISMS-U-57</t>
         </is>
       </c>
       <c r="E164" s="8" t="inlineStr">
@@ -14037,7 +14037,7 @@
       </c>
       <c r="D165" s="6" t="inlineStr">
         <is>
-          <t>U-58</t>
+          <t>ISMS-U-58</t>
         </is>
       </c>
       <c r="E165" s="8" t="inlineStr">
@@ -14100,7 +14100,7 @@
       </c>
       <c r="D166" s="6" t="inlineStr">
         <is>
-          <t>U-59</t>
+          <t>ISMS-U-59</t>
         </is>
       </c>
       <c r="E166" s="8" t="inlineStr">
@@ -14194,7 +14194,7 @@
       </c>
       <c r="D167" s="6" t="inlineStr">
         <is>
-          <t>U-60</t>
+          <t>ISMS-U-60</t>
         </is>
       </c>
       <c r="E167" s="8" t="inlineStr">
@@ -14280,7 +14280,7 @@
       </c>
       <c r="D168" s="6" t="inlineStr">
         <is>
-          <t>U-61</t>
+          <t>ISMS-U-61</t>
         </is>
       </c>
       <c r="E168" s="8" t="inlineStr">
@@ -14358,7 +14358,7 @@
       </c>
       <c r="D169" s="6" t="inlineStr">
         <is>
-          <t>U-62</t>
+          <t>ISMS-U-62</t>
         </is>
       </c>
       <c r="E169" s="8" t="inlineStr">
@@ -14502,7 +14502,7 @@
       </c>
       <c r="D170" s="6" t="inlineStr">
         <is>
-          <t>U-63</t>
+          <t>ISMS-U-63</t>
         </is>
       </c>
       <c r="E170" s="8" t="inlineStr">
@@ -14569,7 +14569,7 @@
       </c>
       <c r="D171" s="6" t="inlineStr">
         <is>
-          <t>U-65</t>
+          <t>ISMS-U-65</t>
         </is>
       </c>
       <c r="E171" s="8" t="inlineStr">
@@ -14678,7 +14678,7 @@
       </c>
       <c r="D172" s="6" t="inlineStr">
         <is>
-          <t>U-66</t>
+          <t>ISMS-U-66</t>
         </is>
       </c>
       <c r="E172" s="8" t="inlineStr">
@@ -14738,7 +14738,7 @@
       </c>
       <c r="D173" s="6" t="inlineStr">
         <is>
-          <t>U-67</t>
+          <t>ISMS-U-67</t>
         </is>
       </c>
       <c r="E173" s="8" t="inlineStr">
@@ -14812,7 +14812,7 @@
       </c>
       <c r="D175" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-01 / W-01</t>
+          <t>CSAP-Windows-01 / ISMS-W-01</t>
         </is>
       </c>
       <c r="E175" s="8" t="inlineStr">
@@ -14899,7 +14899,7 @@
       </c>
       <c r="D176" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-02 / W-02</t>
+          <t>CSAP-Windows-02 / ISMS-W-02</t>
         </is>
       </c>
       <c r="E176" s="8" t="inlineStr">
@@ -14990,7 +14990,7 @@
       </c>
       <c r="D177" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-03 / W-03</t>
+          <t>CSAP-Windows-03 / ISMS-W-03</t>
         </is>
       </c>
       <c r="E177" s="8" t="inlineStr">
@@ -15081,7 +15081,7 @@
       </c>
       <c r="D178" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-04 / W-04</t>
+          <t>CSAP-Windows-04 / ISMS-W-04</t>
         </is>
       </c>
       <c r="E178" s="8" t="inlineStr">
@@ -15174,7 +15174,7 @@
       </c>
       <c r="D179" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-07 / W-05</t>
+          <t>CSAP-Windows-07 / ISMS-W-05</t>
         </is>
       </c>
       <c r="E179" s="8" t="inlineStr">
@@ -15263,7 +15263,7 @@
       </c>
       <c r="D180" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-08 / W-06</t>
+          <t>CSAP-Windows-08 / ISMS-W-06</t>
         </is>
       </c>
       <c r="E180" s="8" t="inlineStr">
@@ -15358,7 +15358,7 @@
       </c>
       <c r="D181" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-09 / W-16</t>
+          <t>CSAP-Windows-09 / ISMS-W-16</t>
         </is>
       </c>
       <c r="E181" s="8" t="inlineStr">
@@ -15462,7 +15462,7 @@
       </c>
       <c r="D182" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-10 / W-17</t>
+          <t>CSAP-Windows-10 / ISMS-W-17</t>
         </is>
       </c>
       <c r="E182" s="8" t="inlineStr">
@@ -15579,7 +15579,7 @@
       </c>
       <c r="D183" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-11 / W-18</t>
+          <t>CSAP-Windows-11 / ISMS-W-18</t>
         </is>
       </c>
       <c r="E183" s="8" t="inlineStr">
@@ -15854,7 +15854,7 @@
       </c>
       <c r="D184" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-12 / W-20</t>
+          <t>CSAP-Windows-12 / ISMS-W-20</t>
         </is>
       </c>
       <c r="E184" s="8" t="inlineStr">
@@ -15959,7 +15959,7 @@
       </c>
       <c r="D185" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-14 / W-22</t>
+          <t>CSAP-Windows-14 / ISMS-W-22</t>
         </is>
       </c>
       <c r="E185" s="8" t="inlineStr">
@@ -16053,7 +16053,7 @@
       </c>
       <c r="D186" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-16 / W-24</t>
+          <t>CSAP-Windows-16 / ISMS-W-24</t>
         </is>
       </c>
       <c r="E186" s="8" t="inlineStr">
@@ -16149,7 +16149,7 @@
       </c>
       <c r="D187" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-17 / W-25</t>
+          <t>CSAP-Windows-17 / ISMS-W-25</t>
         </is>
       </c>
       <c r="E187" s="8" t="inlineStr">
@@ -16260,7 +16260,7 @@
       </c>
       <c r="D188" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-18 / W-26</t>
+          <t>CSAP-Windows-18 / ISMS-W-26</t>
         </is>
       </c>
       <c r="E188" s="8" t="inlineStr">
@@ -16373,7 +16373,7 @@
       </c>
       <c r="D189" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-20 / W-27</t>
+          <t>CSAP-Windows-20 / ISMS-W-27</t>
         </is>
       </c>
       <c r="E189" s="8" t="inlineStr">
@@ -16480,7 +16480,7 @@
       </c>
       <c r="D190" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-21 / W-39</t>
+          <t>CSAP-Windows-21 / ISMS-W-39</t>
         </is>
       </c>
       <c r="E190" s="8" t="inlineStr">
@@ -16568,7 +16568,7 @@
       </c>
       <c r="D191" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-23 / W-44</t>
+          <t>CSAP-Windows-23 / ISMS-W-44</t>
         </is>
       </c>
       <c r="E191" s="8" t="inlineStr">
@@ -16666,7 +16666,7 @@
       </c>
       <c r="D192" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-24 / W-45</t>
+          <t>CSAP-Windows-24 / ISMS-W-45</t>
         </is>
       </c>
       <c r="E192" s="8" t="inlineStr">
@@ -16730,7 +16730,7 @@
       </c>
       <c r="D193" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-25 / W-46</t>
+          <t>CSAP-Windows-25 / ISMS-W-46</t>
         </is>
       </c>
       <c r="E193" s="8" t="inlineStr">
@@ -16814,7 +16814,7 @@
       </c>
       <c r="D194" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-26 / W-48</t>
+          <t>CSAP-Windows-26 / ISMS-W-48</t>
         </is>
       </c>
       <c r="E194" s="8" t="inlineStr">
@@ -16917,7 +16917,7 @@
       </c>
       <c r="D195" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-27 / W-49</t>
+          <t>CSAP-Windows-27 / ISMS-W-49</t>
         </is>
       </c>
       <c r="E195" s="8" t="inlineStr">
@@ -17012,7 +17012,7 @@
       </c>
       <c r="D196" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-28 / W-50</t>
+          <t>CSAP-Windows-28 / ISMS-W-50</t>
         </is>
       </c>
       <c r="E196" s="8" t="inlineStr">
@@ -17109,7 +17109,7 @@
       </c>
       <c r="D197" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-29 / W-51</t>
+          <t>CSAP-Windows-29 / ISMS-W-51</t>
         </is>
       </c>
       <c r="E197" s="8" t="inlineStr">
@@ -17217,7 +17217,7 @@
       </c>
       <c r="D198" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-30 / W-52</t>
+          <t>CSAP-Windows-30 / ISMS-W-52</t>
         </is>
       </c>
       <c r="E198" s="8" t="inlineStr">
@@ -17302,7 +17302,7 @@
       </c>
       <c r="D199" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-31 / W-53</t>
+          <t>CSAP-Windows-31 / ISMS-W-53</t>
         </is>
       </c>
       <c r="E199" s="8" t="inlineStr">
@@ -17399,7 +17399,7 @@
       </c>
       <c r="D200" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-05</t>
+          <t>CSAP-Windows-05</t>
         </is>
       </c>
       <c r="E200" s="8" t="inlineStr">
@@ -17460,7 +17460,7 @@
       </c>
       <c r="D201" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-06</t>
+          <t>CSAP-Windows-06</t>
         </is>
       </c>
       <c r="E201" s="8" t="inlineStr">
@@ -17524,7 +17524,7 @@
       </c>
       <c r="D202" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-13</t>
+          <t>CSAP-Windows-13</t>
         </is>
       </c>
       <c r="E202" s="8" t="inlineStr">
@@ -17583,7 +17583,7 @@
       </c>
       <c r="D203" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-15</t>
+          <t>CSAP-Windows-15</t>
         </is>
       </c>
       <c r="E203" s="8" t="inlineStr">
@@ -17636,7 +17636,7 @@
       </c>
       <c r="D204" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-19</t>
+          <t>CSAP-Windows-19</t>
         </is>
       </c>
       <c r="E204" s="8" t="inlineStr">
@@ -17709,7 +17709,7 @@
       </c>
       <c r="D205" s="6" t="inlineStr">
         <is>
-          <t>CLD-Windows-22</t>
+          <t>CSAP-Windows-22</t>
         </is>
       </c>
       <c r="E205" s="8" t="inlineStr">
@@ -17813,7 +17813,7 @@
       </c>
       <c r="D206" s="6" t="inlineStr">
         <is>
-          <t>W-08</t>
+          <t>ISMS-W-08</t>
         </is>
       </c>
       <c r="E206" s="8" t="inlineStr">
@@ -17883,7 +17883,7 @@
       </c>
       <c r="D207" s="6" t="inlineStr">
         <is>
-          <t>W-09</t>
+          <t>ISMS-W-09</t>
         </is>
       </c>
       <c r="E207" s="8" t="inlineStr">
@@ -17980,7 +17980,7 @@
       </c>
       <c r="D208" s="6" t="inlineStr">
         <is>
-          <t>W-10</t>
+          <t>ISMS-W-10</t>
         </is>
       </c>
       <c r="E208" s="8" t="inlineStr">
@@ -18060,7 +18060,7 @@
       </c>
       <c r="D209" s="6" t="inlineStr">
         <is>
-          <t>W-11</t>
+          <t>ISMS-W-11</t>
         </is>
       </c>
       <c r="E209" s="8" t="inlineStr">
@@ -18122,7 +18122,7 @@
       </c>
       <c r="D210" s="6" t="inlineStr">
         <is>
-          <t>W-12</t>
+          <t>ISMS-W-12</t>
         </is>
       </c>
       <c r="E210" s="8" t="inlineStr">
@@ -18187,7 +18187,7 @@
       </c>
       <c r="D211" s="6" t="inlineStr">
         <is>
-          <t>W-13</t>
+          <t>ISMS-W-13</t>
         </is>
       </c>
       <c r="E211" s="8" t="inlineStr">
@@ -18248,7 +18248,7 @@
       </c>
       <c r="D212" s="6" t="inlineStr">
         <is>
-          <t>W-14</t>
+          <t>ISMS-W-14</t>
         </is>
       </c>
       <c r="E212" s="8" t="inlineStr">
@@ -18334,7 +18334,7 @@
       </c>
       <c r="D213" s="6" t="inlineStr">
         <is>
-          <t>W-15</t>
+          <t>ISMS-W-15</t>
         </is>
       </c>
       <c r="E213" s="8" t="inlineStr">
@@ -18400,7 +18400,7 @@
       </c>
       <c r="D214" s="6" t="inlineStr">
         <is>
-          <t>W-19</t>
+          <t>ISMS-W-19</t>
         </is>
       </c>
       <c r="E214" s="8" t="inlineStr">
@@ -18465,7 +18465,7 @@
       </c>
       <c r="D215" s="6" t="inlineStr">
         <is>
-          <t>W-21</t>
+          <t>ISMS-W-21</t>
         </is>
       </c>
       <c r="E215" s="8" t="inlineStr">
@@ -18528,7 +18528,7 @@
       </c>
       <c r="D216" s="6" t="inlineStr">
         <is>
-          <t>W-23</t>
+          <t>ISMS-W-23</t>
         </is>
       </c>
       <c r="E216" s="8" t="inlineStr">
@@ -18599,7 +18599,7 @@
       </c>
       <c r="D217" s="6" t="inlineStr">
         <is>
-          <t>W-28</t>
+          <t>ISMS-W-28</t>
         </is>
       </c>
       <c r="E217" s="8" t="inlineStr">
@@ -18692,7 +18692,7 @@
       </c>
       <c r="D218" s="6" t="inlineStr">
         <is>
-          <t>W-29</t>
+          <t>ISMS-W-29</t>
         </is>
       </c>
       <c r="E218" s="8" t="inlineStr">
@@ -18761,7 +18761,7 @@
       </c>
       <c r="D219" s="6" t="inlineStr">
         <is>
-          <t>W-31</t>
+          <t>ISMS-W-31</t>
         </is>
       </c>
       <c r="E219" s="8" t="inlineStr">
@@ -18826,7 +18826,7 @@
       </c>
       <c r="D220" s="6" t="inlineStr">
         <is>
-          <t>W-32</t>
+          <t>ISMS-W-32</t>
         </is>
       </c>
       <c r="E220" s="8" t="inlineStr">
@@ -18897,7 +18897,7 @@
       </c>
       <c r="D221" s="6" t="inlineStr">
         <is>
-          <t>W-33</t>
+          <t>ISMS-W-33</t>
         </is>
       </c>
       <c r="E221" s="8" t="inlineStr">
@@ -19016,7 +19016,7 @@
       </c>
       <c r="D222" s="6" t="inlineStr">
         <is>
-          <t>W-34</t>
+          <t>ISMS-W-34</t>
         </is>
       </c>
       <c r="E222" s="8" t="inlineStr">
@@ -19089,7 +19089,7 @@
       </c>
       <c r="D223" s="6" t="inlineStr">
         <is>
-          <t>W-35</t>
+          <t>ISMS-W-35</t>
         </is>
       </c>
       <c r="E223" s="8" t="inlineStr">
@@ -19156,7 +19156,7 @@
       </c>
       <c r="D224" s="6" t="inlineStr">
         <is>
-          <t>W-36</t>
+          <t>ISMS-W-36</t>
         </is>
       </c>
       <c r="E224" s="8" t="inlineStr">
@@ -19231,7 +19231,7 @@
       </c>
       <c r="D225" s="6" t="inlineStr">
         <is>
-          <t>W-37</t>
+          <t>ISMS-W-37</t>
         </is>
       </c>
       <c r="E225" s="8" t="inlineStr">
@@ -19299,7 +19299,7 @@
       </c>
       <c r="D226" s="6" t="inlineStr">
         <is>
-          <t>W-38</t>
+          <t>ISMS-W-38</t>
         </is>
       </c>
       <c r="E226" s="8" t="inlineStr">
@@ -19368,7 +19368,7 @@
       </c>
       <c r="D227" s="6" t="inlineStr">
         <is>
-          <t>W-40</t>
+          <t>ISMS-W-40</t>
         </is>
       </c>
       <c r="E227" s="8" t="inlineStr">
@@ -19451,7 +19451,7 @@
       </c>
       <c r="D228" s="6" t="inlineStr">
         <is>
-          <t>W-41</t>
+          <t>ISMS-W-41</t>
         </is>
       </c>
       <c r="E228" s="8" t="inlineStr">
@@ -19538,7 +19538,7 @@
       </c>
       <c r="D229" s="6" t="inlineStr">
         <is>
-          <t>W-42</t>
+          <t>ISMS-W-42</t>
         </is>
       </c>
       <c r="E229" s="8" t="inlineStr">
@@ -19603,7 +19603,7 @@
       </c>
       <c r="D230" s="6" t="inlineStr">
         <is>
-          <t>W-43</t>
+          <t>ISMS-W-43</t>
         </is>
       </c>
       <c r="E230" s="8" t="inlineStr">
@@ -19672,7 +19672,7 @@
       </c>
       <c r="D231" s="6" t="inlineStr">
         <is>
-          <t>W-47</t>
+          <t>ISMS-W-47</t>
         </is>
       </c>
       <c r="E231" s="8" t="inlineStr">
@@ -19755,7 +19755,7 @@
       </c>
       <c r="D232" s="6" t="inlineStr">
         <is>
-          <t>W-54</t>
+          <t>ISMS-W-54</t>
         </is>
       </c>
       <c r="E232" s="8" t="inlineStr">
@@ -19828,7 +19828,7 @@
       </c>
       <c r="D233" s="6" t="inlineStr">
         <is>
-          <t>W-55</t>
+          <t>ISMS-W-55</t>
         </is>
       </c>
       <c r="E233" s="8" t="inlineStr">
@@ -19897,7 +19897,7 @@
       </c>
       <c r="D234" s="6" t="inlineStr">
         <is>
-          <t>W-56</t>
+          <t>ISMS-W-56</t>
         </is>
       </c>
       <c r="E234" s="8" t="inlineStr">
@@ -19975,7 +19975,7 @@
       </c>
       <c r="D235" s="6" t="inlineStr">
         <is>
-          <t>W-57</t>
+          <t>ISMS-W-57</t>
         </is>
       </c>
       <c r="E235" s="8" t="inlineStr">
@@ -20060,7 +20060,7 @@
       </c>
       <c r="D236" s="6" t="inlineStr">
         <is>
-          <t>W-58</t>
+          <t>ISMS-W-58</t>
         </is>
       </c>
       <c r="E236" s="8" t="inlineStr">
@@ -20141,7 +20141,7 @@
       </c>
       <c r="D237" s="6" t="inlineStr">
         <is>
-          <t>W-59</t>
+          <t>ISMS-W-59</t>
         </is>
       </c>
       <c r="E237" s="8" t="inlineStr">
@@ -20213,7 +20213,7 @@
       </c>
       <c r="D238" s="6" t="inlineStr">
         <is>
-          <t>W-60</t>
+          <t>ISMS-W-60</t>
         </is>
       </c>
       <c r="E238" s="8" t="inlineStr">
@@ -20301,7 +20301,7 @@
       </c>
       <c r="D239" s="6" t="inlineStr">
         <is>
-          <t>W-61</t>
+          <t>ISMS-W-61</t>
         </is>
       </c>
       <c r="E239" s="8" t="inlineStr">
@@ -20364,7 +20364,7 @@
       </c>
       <c r="D240" s="6" t="inlineStr">
         <is>
-          <t>W-62</t>
+          <t>ISMS-W-62</t>
         </is>
       </c>
       <c r="E240" s="8" t="inlineStr">
@@ -20433,7 +20433,7 @@
       </c>
       <c r="D241" s="6" t="inlineStr">
         <is>
-          <t>W-63</t>
+          <t>ISMS-W-63</t>
         </is>
       </c>
       <c r="E241" s="8" t="inlineStr">
@@ -20494,7 +20494,7 @@
       </c>
       <c r="D242" s="6" t="inlineStr">
         <is>
-          <t>W-64</t>
+          <t>ISMS-W-64</t>
         </is>
       </c>
       <c r="E242" s="8" t="inlineStr">
@@ -20570,7 +20570,7 @@
       </c>
       <c r="D244" s="6" t="inlineStr">
         <is>
-          <t>CLD-MY-SQL-05 / D-07</t>
+          <t>CSAP-MY-SQL-05 / ISMS-D-07</t>
         </is>
       </c>
       <c r="E244" s="8" t="inlineStr">
@@ -20654,7 +20654,7 @@
       </c>
       <c r="D245" s="6" t="inlineStr">
         <is>
-          <t>CLD-MY-SQL-07 / D-08</t>
+          <t>CSAP-MY-SQL-07 / ISMS-D-08</t>
         </is>
       </c>
       <c r="E245" s="8" t="inlineStr">
@@ -20770,7 +20770,7 @@
       </c>
       <c r="D246" s="6" t="inlineStr">
         <is>
-          <t>CLD-MY-SQL-01</t>
+          <t>CSAP-MY-SQL-01</t>
         </is>
       </c>
       <c r="E246" s="8" t="inlineStr">
@@ -20823,7 +20823,7 @@
       </c>
       <c r="D247" s="6" t="inlineStr">
         <is>
-          <t>CLD-MY-SQL-02</t>
+          <t>CSAP-MY-SQL-02</t>
         </is>
       </c>
       <c r="E247" s="8" t="inlineStr">
@@ -20890,7 +20890,7 @@
       </c>
       <c r="D248" s="6" t="inlineStr">
         <is>
-          <t>CLD-MY-SQL-03</t>
+          <t>CSAP-MY-SQL-03</t>
         </is>
       </c>
       <c r="E248" s="8" t="inlineStr">
@@ -20943,7 +20943,7 @@
       </c>
       <c r="D249" s="6" t="inlineStr">
         <is>
-          <t>CLD-MY-SQL-04</t>
+          <t>CSAP-MY-SQL-04</t>
         </is>
       </c>
       <c r="E249" s="8" t="inlineStr">
@@ -20990,7 +20990,7 @@
       </c>
       <c r="D250" s="6" t="inlineStr">
         <is>
-          <t>CLD-MY-SQL-06</t>
+          <t>CSAP-MY-SQL-06</t>
         </is>
       </c>
       <c r="E250" s="8" t="inlineStr">
@@ -21040,7 +21040,7 @@
       </c>
       <c r="D251" s="6" t="inlineStr">
         <is>
-          <t>CLD-MY-SQL-08</t>
+          <t>CSAP-MY-SQL-08</t>
         </is>
       </c>
       <c r="E251" s="8" t="inlineStr">
@@ -21101,7 +21101,7 @@
       </c>
       <c r="D252" s="6" t="inlineStr">
         <is>
-          <t>CLD-MY-SQL-09</t>
+          <t>CSAP-MY-SQL-09</t>
         </is>
       </c>
       <c r="E252" s="8" t="inlineStr">
@@ -21157,7 +21157,7 @@
       </c>
       <c r="D253" s="6" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>ISMS-D-01</t>
         </is>
       </c>
       <c r="E253" s="8" t="inlineStr">
@@ -21296,7 +21296,7 @@
       </c>
       <c r="D254" s="6" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>ISMS-D-02</t>
         </is>
       </c>
       <c r="E254" s="8" t="inlineStr">
@@ -21359,7 +21359,7 @@
       </c>
       <c r="D255" s="6" t="inlineStr">
         <is>
-          <t>D-03</t>
+          <t>ISMS-D-03</t>
         </is>
       </c>
       <c r="E255" s="8" t="inlineStr">
@@ -21468,7 +21468,7 @@
       </c>
       <c r="D256" s="6" t="inlineStr">
         <is>
-          <t>D-04</t>
+          <t>ISMS-D-04</t>
         </is>
       </c>
       <c r="E256" s="8" t="inlineStr">
@@ -21553,7 +21553,7 @@
       </c>
       <c r="D257" s="6" t="inlineStr">
         <is>
-          <t>D-06</t>
+          <t>ISMS-D-06</t>
         </is>
       </c>
       <c r="E257" s="8" t="inlineStr">
@@ -21630,7 +21630,7 @@
       </c>
       <c r="D258" s="6" t="inlineStr">
         <is>
-          <t>D-10</t>
+          <t>ISMS-D-10</t>
         </is>
       </c>
       <c r="E258" s="8" t="inlineStr">
@@ -21691,7 +21691,7 @@
       </c>
       <c r="D259" s="6" t="inlineStr">
         <is>
-          <t>D-11</t>
+          <t>ISMS-D-11</t>
         </is>
       </c>
       <c r="E259" s="8" t="inlineStr">
@@ -21752,7 +21752,7 @@
       </c>
       <c r="D260" s="6" t="inlineStr">
         <is>
-          <t>D-21</t>
+          <t>ISMS-D-21</t>
         </is>
       </c>
       <c r="E260" s="8" t="inlineStr">
@@ -21817,7 +21817,7 @@
       </c>
       <c r="D261" s="6" t="inlineStr">
         <is>
-          <t>D-25</t>
+          <t>ISMS-D-25</t>
         </is>
       </c>
       <c r="E261" s="8" t="inlineStr">
@@ -21893,7 +21893,7 @@
       </c>
       <c r="D263" s="6" t="inlineStr">
         <is>
-          <t>CLD-MS-SQL-05 / D-24</t>
+          <t>CSAP-MS-SQL-05 / ISMS-D-24</t>
         </is>
       </c>
       <c r="E263" s="8" t="inlineStr">
@@ -22020,7 +22020,7 @@
       </c>
       <c r="D264" s="6" t="inlineStr">
         <is>
-          <t>CLD-MS-SQL-06 / D-23</t>
+          <t>CSAP-MS-SQL-06 / ISMS-D-23</t>
         </is>
       </c>
       <c r="E264" s="8" t="inlineStr">
@@ -22178,7 +22178,7 @@
       </c>
       <c r="D265" s="6" t="inlineStr">
         <is>
-          <t>CLD-MS-SQL-01</t>
+          <t>CSAP-MS-SQL-01</t>
         </is>
       </c>
       <c r="E265" s="8" t="inlineStr">
@@ -22242,7 +22242,7 @@
       </c>
       <c r="D266" s="6" t="inlineStr">
         <is>
-          <t>CLD-MS-SQL-02</t>
+          <t>CSAP-MS-SQL-02</t>
         </is>
       </c>
       <c r="E266" s="8" t="inlineStr">
@@ -22300,7 +22300,7 @@
       </c>
       <c r="D267" s="6" t="inlineStr">
         <is>
-          <t>CLD-MS-SQL-03</t>
+          <t>CSAP-MS-SQL-03</t>
         </is>
       </c>
       <c r="E267" s="8" t="inlineStr">
@@ -22353,7 +22353,7 @@
       </c>
       <c r="D268" s="6" t="inlineStr">
         <is>
-          <t>CLD-MS-SQL-04</t>
+          <t>CSAP-MS-SQL-04</t>
         </is>
       </c>
       <c r="E268" s="8" t="inlineStr">
@@ -22405,7 +22405,7 @@
       </c>
       <c r="D269" s="6" t="inlineStr">
         <is>
-          <t>CLD-MS-SQL-07</t>
+          <t>CSAP-MS-SQL-07</t>
         </is>
       </c>
       <c r="E269" s="8" t="inlineStr">
@@ -22468,7 +22468,7 @@
       </c>
       <c r="D270" s="6" t="inlineStr">
         <is>
-          <t>CLD-MS-SQL-08</t>
+          <t>CSAP-MS-SQL-08</t>
         </is>
       </c>
       <c r="E270" s="8" t="inlineStr">
@@ -22520,7 +22520,7 @@
       </c>
       <c r="D271" s="6" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>ISMS-D-01</t>
         </is>
       </c>
       <c r="E271" s="8" t="inlineStr">
@@ -22581,7 +22581,7 @@
       </c>
       <c r="D272" s="6" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>ISMS-D-02</t>
         </is>
       </c>
       <c r="E272" s="8" t="inlineStr">
@@ -22638,7 +22638,7 @@
       </c>
       <c r="D273" s="6" t="inlineStr">
         <is>
-          <t>D-03</t>
+          <t>ISMS-D-03</t>
         </is>
       </c>
       <c r="E273" s="8" t="inlineStr">
@@ -22709,7 +22709,7 @@
       </c>
       <c r="D274" s="6" t="inlineStr">
         <is>
-          <t>D-04</t>
+          <t>ISMS-D-04</t>
         </is>
       </c>
       <c r="E274" s="8" t="inlineStr">
@@ -22770,7 +22770,7 @@
       </c>
       <c r="D275" s="6" t="inlineStr">
         <is>
-          <t>D-06</t>
+          <t>ISMS-D-06</t>
         </is>
       </c>
       <c r="E275" s="8" t="inlineStr">
@@ -22843,7 +22843,7 @@
       </c>
       <c r="D276" s="6" t="inlineStr">
         <is>
-          <t>D-08</t>
+          <t>ISMS-D-08</t>
         </is>
       </c>
       <c r="E276" s="8" t="inlineStr">
@@ -22928,7 +22928,7 @@
       </c>
       <c r="D277" s="6" t="inlineStr">
         <is>
-          <t>D-11</t>
+          <t>ISMS-D-11</t>
         </is>
       </c>
       <c r="E277" s="8" t="inlineStr">
@@ -22991,7 +22991,7 @@
       </c>
       <c r="D278" s="6" t="inlineStr">
         <is>
-          <t>D-16</t>
+          <t>ISMS-D-16</t>
         </is>
       </c>
       <c r="E278" s="8" t="inlineStr">
@@ -23057,7 +23057,7 @@
       </c>
       <c r="D279" s="6" t="inlineStr">
         <is>
-          <t>D-25</t>
+          <t>ISMS-D-25</t>
         </is>
       </c>
       <c r="E279" s="8" t="inlineStr">
@@ -23126,7 +23126,7 @@
       </c>
       <c r="D280" s="6" t="inlineStr">
         <is>
-          <t>D-26</t>
+          <t>ISMS-D-26</t>
         </is>
       </c>
       <c r="E280" s="8" t="inlineStr">
@@ -23214,7 +23214,7 @@
       </c>
       <c r="D282" s="6" t="inlineStr">
         <is>
-          <t>CLD-Redis-01</t>
+          <t>CSAP-Redis-01</t>
         </is>
       </c>
       <c r="E282" s="8" t="inlineStr">
@@ -23264,7 +23264,7 @@
       </c>
       <c r="D283" s="6" t="inlineStr">
         <is>
-          <t>CLD-Redis-02</t>
+          <t>CSAP-Redis-02</t>
         </is>
       </c>
       <c r="E283" s="8" t="inlineStr">
@@ -23316,7 +23316,7 @@
       </c>
       <c r="D284" s="6" t="inlineStr">
         <is>
-          <t>CLD-Redis-03</t>
+          <t>CSAP-Redis-03</t>
         </is>
       </c>
       <c r="E284" s="8" t="inlineStr">
@@ -23363,7 +23363,7 @@
       </c>
       <c r="D285" s="6" t="inlineStr">
         <is>
-          <t>CLD-Redis-04</t>
+          <t>CSAP-Redis-04</t>
         </is>
       </c>
       <c r="E285" s="8" t="inlineStr">
@@ -23417,7 +23417,7 @@
       </c>
       <c r="D286" s="6" t="inlineStr">
         <is>
-          <t>CLD-Redis-05</t>
+          <t>CSAP-Redis-05</t>
         </is>
       </c>
       <c r="E286" s="8" t="inlineStr">
@@ -23464,7 +23464,7 @@
       </c>
       <c r="D287" s="6" t="inlineStr">
         <is>
-          <t>CLD-Redis-06</t>
+          <t>CSAP-Redis-06</t>
         </is>
       </c>
       <c r="E287" s="8" t="inlineStr">
@@ -23515,7 +23515,7 @@
       </c>
       <c r="D288" s="6" t="inlineStr">
         <is>
-          <t>CLD-Redis-07</t>
+          <t>CSAP-Redis-07</t>
         </is>
       </c>
       <c r="E288" s="8" t="inlineStr">
@@ -23569,7 +23569,7 @@
       </c>
       <c r="D289" s="6" t="inlineStr">
         <is>
-          <t>CLD-Redis-08</t>
+          <t>CSAP-Redis-08</t>
         </is>
       </c>
       <c r="E289" s="8" t="inlineStr">
@@ -23638,7 +23638,7 @@
       </c>
       <c r="D291" s="6" t="inlineStr">
         <is>
-          <t>CLD-Elasticsearch-01</t>
+          <t>CSAP-Elasticsearch-01</t>
         </is>
       </c>
       <c r="E291" s="8" t="inlineStr">
@@ -23721,7 +23721,7 @@
       </c>
       <c r="D292" s="6" t="inlineStr">
         <is>
-          <t>CLD-Elasticsearch-02</t>
+          <t>CSAP-Elasticsearch-02</t>
         </is>
       </c>
       <c r="E292" s="8" t="inlineStr">
@@ -23786,7 +23786,7 @@
       </c>
       <c r="D293" s="6" t="inlineStr">
         <is>
-          <t>CLD-Elasticsearch-03</t>
+          <t>CSAP-Elasticsearch-03</t>
         </is>
       </c>
       <c r="E293" s="8" t="inlineStr">
@@ -23851,7 +23851,7 @@
       </c>
       <c r="D294" s="6" t="inlineStr">
         <is>
-          <t>CLD-Elasticsearch-04</t>
+          <t>CSAP-Elasticsearch-04</t>
         </is>
       </c>
       <c r="E294" s="8" t="inlineStr">
@@ -23902,7 +23902,7 @@
       </c>
       <c r="D295" s="6" t="inlineStr">
         <is>
-          <t>CLD-Elasticsearch-05</t>
+          <t>CSAP-Elasticsearch-05</t>
         </is>
       </c>
       <c r="E295" s="8" t="inlineStr">
@@ -23952,7 +23952,7 @@
       </c>
       <c r="D296" s="6" t="inlineStr">
         <is>
-          <t>CLD-Elasticsearch-06</t>
+          <t>CSAP-Elasticsearch-06</t>
         </is>
       </c>
       <c r="E296" s="8" t="inlineStr">
@@ -24002,7 +24002,7 @@
       </c>
       <c r="D297" s="6" t="inlineStr">
         <is>
-          <t>CLD-Elasticsearch-07</t>
+          <t>CSAP-Elasticsearch-07</t>
         </is>
       </c>
       <c r="E297" s="8" t="inlineStr">
@@ -24054,7 +24054,7 @@
       </c>
       <c r="D298" s="6" t="inlineStr">
         <is>
-          <t>CLD-Elasticsearch-08</t>
+          <t>CSAP-Elasticsearch-08</t>
         </is>
       </c>
       <c r="E298" s="8" t="inlineStr">
@@ -24106,7 +24106,7 @@
       </c>
       <c r="D299" s="6" t="inlineStr">
         <is>
-          <t>CLD-Elasticsearch-09</t>
+          <t>CSAP-Elasticsearch-09</t>
         </is>
       </c>
       <c r="E299" s="8" t="inlineStr">
@@ -24161,7 +24161,7 @@
       </c>
       <c r="D300" s="6" t="inlineStr">
         <is>
-          <t>CLD-Elasticsearch-10</t>
+          <t>CSAP-Elasticsearch-10</t>
         </is>
       </c>
       <c r="E300" s="8" t="inlineStr">
@@ -24233,7 +24233,7 @@
       </c>
       <c r="D302" s="6" t="inlineStr">
         <is>
-          <t>CLD-MongoDB-01</t>
+          <t>CSAP-MongoDB-01</t>
         </is>
       </c>
       <c r="E302" s="8" t="inlineStr">
@@ -24290,7 +24290,7 @@
       </c>
       <c r="D303" s="6" t="inlineStr">
         <is>
-          <t>CLD-MongoDB-02</t>
+          <t>CSAP-MongoDB-02</t>
         </is>
       </c>
       <c r="E303" s="8" t="inlineStr">
@@ -24339,7 +24339,7 @@
       </c>
       <c r="D304" s="6" t="inlineStr">
         <is>
-          <t>CLD-MongoDB-03</t>
+          <t>CSAP-MongoDB-03</t>
         </is>
       </c>
       <c r="E304" s="8" t="inlineStr">
@@ -24396,7 +24396,7 @@
       </c>
       <c r="D305" s="6" t="inlineStr">
         <is>
-          <t>CLD-MongoDB-04</t>
+          <t>CSAP-MongoDB-04</t>
         </is>
       </c>
       <c r="E305" s="8" t="inlineStr">
@@ -24458,7 +24458,7 @@
       </c>
       <c r="D306" s="6" t="inlineStr">
         <is>
-          <t>CLD-MongoDB-05</t>
+          <t>CSAP-MongoDB-05</t>
         </is>
       </c>
       <c r="E306" s="8" t="inlineStr">
@@ -24516,7 +24516,7 @@
       </c>
       <c r="D307" s="6" t="inlineStr">
         <is>
-          <t>CLD-MongoDB-06</t>
+          <t>CSAP-MongoDB-06</t>
         </is>
       </c>
       <c r="E307" s="8" t="inlineStr">
@@ -24576,7 +24576,7 @@
       </c>
       <c r="D308" s="6" t="inlineStr">
         <is>
-          <t>CLD-MongoDB-07</t>
+          <t>CSAP-MongoDB-07</t>
         </is>
       </c>
       <c r="E308" s="8" t="inlineStr">
@@ -24629,7 +24629,7 @@
       </c>
       <c r="D309" s="6" t="inlineStr">
         <is>
-          <t>CLD-MongoDB-08</t>
+          <t>CSAP-MongoDB-08</t>
         </is>
       </c>
       <c r="E309" s="8" t="inlineStr">
@@ -24683,7 +24683,7 @@
       </c>
       <c r="D310" s="6" t="inlineStr">
         <is>
-          <t>CLD-MongoDB-09</t>
+          <t>CSAP-MongoDB-09</t>
         </is>
       </c>
       <c r="E310" s="8" t="inlineStr">
@@ -24750,7 +24750,7 @@
       </c>
       <c r="D312" s="6" t="inlineStr">
         <is>
-          <t>CLD-PostgreSQL-07 / D-08</t>
+          <t>CSAP-PostgreSQL-07 / ISMS-D-08</t>
         </is>
       </c>
       <c r="E312" s="8" t="inlineStr">
@@ -24846,7 +24846,7 @@
       </c>
       <c r="D313" s="6" t="inlineStr">
         <is>
-          <t>CLD-PostgreSQL-01</t>
+          <t>CSAP-PostgreSQL-01</t>
         </is>
       </c>
       <c r="E313" s="8" t="inlineStr">
@@ -24900,7 +24900,7 @@
       </c>
       <c r="D314" s="6" t="inlineStr">
         <is>
-          <t>CLD-PostgreSQL-02</t>
+          <t>CSAP-PostgreSQL-02</t>
         </is>
       </c>
       <c r="E314" s="8" t="inlineStr">
@@ -24960,7 +24960,7 @@
       </c>
       <c r="D315" s="6" t="inlineStr">
         <is>
-          <t>CLD-PostgreSQL-03</t>
+          <t>CSAP-PostgreSQL-03</t>
         </is>
       </c>
       <c r="E315" s="8" t="inlineStr">
@@ -25013,7 +25013,7 @@
       </c>
       <c r="D316" s="6" t="inlineStr">
         <is>
-          <t>CLD-PostgreSQL-04</t>
+          <t>CSAP-PostgreSQL-04</t>
         </is>
       </c>
       <c r="E316" s="8" t="inlineStr">
@@ -25064,7 +25064,7 @@
       </c>
       <c r="D317" s="6" t="inlineStr">
         <is>
-          <t>CLD-PostgreSQL-05</t>
+          <t>CSAP-PostgreSQL-05</t>
         </is>
       </c>
       <c r="E317" s="8" t="inlineStr">
@@ -25125,7 +25125,7 @@
       </c>
       <c r="D318" s="6" t="inlineStr">
         <is>
-          <t>CLD-PostgreSQL-06</t>
+          <t>CSAP-PostgreSQL-06</t>
         </is>
       </c>
       <c r="E318" s="8" t="inlineStr">
@@ -25173,7 +25173,7 @@
       </c>
       <c r="D319" s="6" t="inlineStr">
         <is>
-          <t>CLD-PostgreSQL-08</t>
+          <t>CSAP-PostgreSQL-08</t>
         </is>
       </c>
       <c r="E319" s="8" t="inlineStr">
@@ -25219,7 +25219,7 @@
       </c>
       <c r="D320" s="6" t="inlineStr">
         <is>
-          <t>CLD-PostgreSQL-09</t>
+          <t>CSAP-PostgreSQL-09</t>
         </is>
       </c>
       <c r="E320" s="8" t="inlineStr">
@@ -25267,7 +25267,7 @@
       </c>
       <c r="D321" s="6" t="inlineStr">
         <is>
-          <t>CLD-PostgreSQL-10</t>
+          <t>CSAP-PostgreSQL-10</t>
         </is>
       </c>
       <c r="E321" s="8" t="inlineStr">
@@ -25326,7 +25326,7 @@
       </c>
       <c r="D322" s="6" t="inlineStr">
         <is>
-          <t>CLD-PostgreSQL-11</t>
+          <t>CSAP-PostgreSQL-11</t>
         </is>
       </c>
       <c r="E322" s="8" t="inlineStr">
@@ -25377,7 +25377,7 @@
       </c>
       <c r="D323" s="6" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>ISMS-D-01</t>
         </is>
       </c>
       <c r="E323" s="8" t="inlineStr">
@@ -25438,7 +25438,7 @@
       </c>
       <c r="D324" s="6" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>ISMS-D-02</t>
         </is>
       </c>
       <c r="E324" s="8" t="inlineStr">
@@ -25503,7 +25503,7 @@
       </c>
       <c r="D325" s="6" t="inlineStr">
         <is>
-          <t>D-03</t>
+          <t>ISMS-D-03</t>
         </is>
       </c>
       <c r="E325" s="8" t="inlineStr">
@@ -25730,7 +25730,7 @@
       </c>
       <c r="D326" s="6" t="inlineStr">
         <is>
-          <t>D-04</t>
+          <t>ISMS-D-04</t>
         </is>
       </c>
       <c r="E326" s="8" t="inlineStr">
@@ -25807,7 +25807,7 @@
       </c>
       <c r="D327" s="6" t="inlineStr">
         <is>
-          <t>D-06</t>
+          <t>ISMS-D-06</t>
         </is>
       </c>
       <c r="E327" s="8" t="inlineStr">
@@ -25884,7 +25884,7 @@
       </c>
       <c r="D328" s="6" t="inlineStr">
         <is>
-          <t>D-10</t>
+          <t>ISMS-D-10</t>
         </is>
       </c>
       <c r="E328" s="8" t="inlineStr">
@@ -25969,7 +25969,7 @@
       </c>
       <c r="D329" s="6" t="inlineStr">
         <is>
-          <t>D-11</t>
+          <t>ISMS-D-11</t>
         </is>
       </c>
       <c r="E329" s="8" t="inlineStr">
@@ -26034,7 +26034,7 @@
       </c>
       <c r="D330" s="6" t="inlineStr">
         <is>
-          <t>D-14</t>
+          <t>ISMS-D-14</t>
         </is>
       </c>
       <c r="E330" s="8" t="inlineStr">
@@ -26124,7 +26124,7 @@
       </c>
       <c r="D331" s="6" t="inlineStr">
         <is>
-          <t>D-20</t>
+          <t>ISMS-D-20</t>
         </is>
       </c>
       <c r="E331" s="8" t="inlineStr">
@@ -26187,7 +26187,7 @@
       </c>
       <c r="D332" s="6" t="inlineStr">
         <is>
-          <t>D-25</t>
+          <t>ISMS-D-25</t>
         </is>
       </c>
       <c r="E332" s="8" t="inlineStr">
@@ -26250,7 +26250,7 @@
       </c>
       <c r="D333" s="6" t="inlineStr">
         <is>
-          <t>D-26</t>
+          <t>ISMS-D-26</t>
         </is>
       </c>
       <c r="E333" s="8" t="inlineStr">
@@ -26332,7 +26332,7 @@
       </c>
       <c r="D335" s="6" t="inlineStr">
         <is>
-          <t>CLD-Apache-01 / WEB-11</t>
+          <t>CSAP-Apache-01 / ISMS-WEB-11</t>
         </is>
       </c>
       <c r="E335" s="8" t="inlineStr">
@@ -26404,7 +26404,7 @@
       </c>
       <c r="D336" s="6" t="inlineStr">
         <is>
-          <t>CLD-Apache-02 / WEB-07</t>
+          <t>CSAP-Apache-02 / ISMS-WEB-07</t>
         </is>
       </c>
       <c r="E336" s="8" t="inlineStr">
@@ -26483,7 +26483,7 @@
       </c>
       <c r="D337" s="6" t="inlineStr">
         <is>
-          <t>CLD-Apache-03 / WEB-12</t>
+          <t>CSAP-Apache-03 / ISMS-WEB-12</t>
         </is>
       </c>
       <c r="E337" s="8" t="inlineStr">
@@ -26566,7 +26566,7 @@
       </c>
       <c r="D338" s="6" t="inlineStr">
         <is>
-          <t>CLD-Apache-04 / WEB-08</t>
+          <t>CSAP-Apache-04 / ISMS-WEB-08</t>
         </is>
       </c>
       <c r="E338" s="8" t="inlineStr">
@@ -26641,7 +26641,7 @@
       </c>
       <c r="D339" s="6" t="inlineStr">
         <is>
-          <t>CLD-Apache-05 / WEB-04</t>
+          <t>CSAP-Apache-05 / ISMS-WEB-04</t>
         </is>
       </c>
       <c r="E339" s="8" t="inlineStr">
@@ -26729,7 +26729,7 @@
       </c>
       <c r="D340" s="6" t="inlineStr">
         <is>
-          <t>CLD-Apache-06 / WEB-09</t>
+          <t>CSAP-Apache-06 / ISMS-WEB-09</t>
         </is>
       </c>
       <c r="E340" s="8" t="inlineStr">
@@ -26823,7 +26823,7 @@
       </c>
       <c r="D341" s="6" t="inlineStr">
         <is>
-          <t>CLD-Apache-07</t>
+          <t>CSAP-Apache-07</t>
         </is>
       </c>
       <c r="E341" s="8" t="inlineStr">
@@ -26874,7 +26874,7 @@
       </c>
       <c r="D342" s="6" t="inlineStr">
         <is>
-          <t>WEB-05</t>
+          <t>ISMS-WEB-05</t>
         </is>
       </c>
       <c r="E342" s="8" t="inlineStr">
@@ -26949,7 +26949,7 @@
       </c>
       <c r="D343" s="6" t="inlineStr">
         <is>
-          <t>WEB-06</t>
+          <t>ISMS-WEB-06</t>
         </is>
       </c>
       <c r="E343" s="8" t="inlineStr">
@@ -27072,7 +27072,7 @@
       </c>
       <c r="D344" s="6" t="inlineStr">
         <is>
-          <t>WEB-10</t>
+          <t>ISMS-WEB-10</t>
         </is>
       </c>
       <c r="E344" s="8" t="inlineStr">
@@ -27141,7 +27141,7 @@
       </c>
       <c r="D345" s="6" t="inlineStr">
         <is>
-          <t>WEB-14</t>
+          <t>ISMS-WEB-14</t>
         </is>
       </c>
       <c r="E345" s="8" t="inlineStr">
@@ -27200,7 +27200,7 @@
       </c>
       <c r="D346" s="6" t="inlineStr">
         <is>
-          <t>WEB-16</t>
+          <t>ISMS-WEB-16</t>
         </is>
       </c>
       <c r="E346" s="8" t="inlineStr">
@@ -27303,7 +27303,7 @@
       </c>
       <c r="D347" s="6" t="inlineStr">
         <is>
-          <t>WEB-17</t>
+          <t>ISMS-WEB-17</t>
         </is>
       </c>
       <c r="E347" s="8" t="inlineStr">
@@ -27378,7 +27378,7 @@
       </c>
       <c r="D348" s="6" t="inlineStr">
         <is>
-          <t>WEB-18</t>
+          <t>ISMS-WEB-18</t>
         </is>
       </c>
       <c r="E348" s="8" t="inlineStr">
@@ -27455,7 +27455,7 @@
       </c>
       <c r="D349" s="6" t="inlineStr">
         <is>
-          <t>WEB-19</t>
+          <t>ISMS-WEB-19</t>
         </is>
       </c>
       <c r="E349" s="8" t="inlineStr">
@@ -27530,7 +27530,7 @@
       </c>
       <c r="D350" s="6" t="inlineStr">
         <is>
-          <t>WEB-20</t>
+          <t>ISMS-WEB-20</t>
         </is>
       </c>
       <c r="E350" s="8" t="inlineStr">
@@ -27621,7 +27621,7 @@
       </c>
       <c r="D351" s="6" t="inlineStr">
         <is>
-          <t>WEB-21</t>
+          <t>ISMS-WEB-21</t>
         </is>
       </c>
       <c r="E351" s="8" t="inlineStr">
@@ -27728,7 +27728,7 @@
       </c>
       <c r="D352" s="6" t="inlineStr">
         <is>
-          <t>WEB-22</t>
+          <t>ISMS-WEB-22</t>
         </is>
       </c>
       <c r="E352" s="8" t="inlineStr">
@@ -27799,7 +27799,7 @@
       </c>
       <c r="D353" s="6" t="inlineStr">
         <is>
-          <t>WEB-24</t>
+          <t>ISMS-WEB-24</t>
         </is>
       </c>
       <c r="E353" s="8" t="inlineStr">
@@ -27893,7 +27893,7 @@
       </c>
       <c r="D354" s="6" t="inlineStr">
         <is>
-          <t>WEB-25</t>
+          <t>ISMS-WEB-25</t>
         </is>
       </c>
       <c r="E354" s="8" t="inlineStr">
@@ -27959,7 +27959,7 @@
       </c>
       <c r="D355" s="6" t="inlineStr">
         <is>
-          <t>WEB-26</t>
+          <t>ISMS-WEB-26</t>
         </is>
       </c>
       <c r="E355" s="8" t="inlineStr">
@@ -28035,7 +28035,7 @@
       </c>
       <c r="D357" s="6" t="inlineStr">
         <is>
-          <t>CLD-Nginx-01 / WEB-11</t>
+          <t>CSAP-Nginx-01 / ISMS-WEB-11</t>
         </is>
       </c>
       <c r="E357" s="8" t="inlineStr">
@@ -28109,7 +28109,7 @@
       </c>
       <c r="D358" s="6" t="inlineStr">
         <is>
-          <t>CLD-Nginx-02 / WEB-07</t>
+          <t>CSAP-Nginx-02 / ISMS-WEB-07</t>
         </is>
       </c>
       <c r="E358" s="8" t="inlineStr">
@@ -28183,7 +28183,7 @@
       </c>
       <c r="D359" s="6" t="inlineStr">
         <is>
-          <t>CLD-Nginx-03 / WEB-12</t>
+          <t>CSAP-Nginx-03 / ISMS-WEB-12</t>
         </is>
       </c>
       <c r="E359" s="8" t="inlineStr">
@@ -28262,7 +28262,7 @@
       </c>
       <c r="D360" s="6" t="inlineStr">
         <is>
-          <t>CLD-Nginx-04 / WEB-08</t>
+          <t>CSAP-Nginx-04 / ISMS-WEB-08</t>
         </is>
       </c>
       <c r="E360" s="8" t="inlineStr">
@@ -28342,7 +28342,7 @@
       </c>
       <c r="D361" s="6" t="inlineStr">
         <is>
-          <t>CLD-Nginx-05 / WEB-04</t>
+          <t>CSAP-Nginx-05 / ISMS-WEB-04</t>
         </is>
       </c>
       <c r="E361" s="8" t="inlineStr">
@@ -28421,7 +28421,7 @@
       </c>
       <c r="D362" s="6" t="inlineStr">
         <is>
-          <t>CLD-Nginx-06 / WEB-09</t>
+          <t>CSAP-Nginx-06 / ISMS-WEB-09</t>
         </is>
       </c>
       <c r="E362" s="8" t="inlineStr">
@@ -28514,7 +28514,7 @@
       </c>
       <c r="D363" s="6" t="inlineStr">
         <is>
-          <t>CLD-Nginx-07</t>
+          <t>CSAP-Nginx-07</t>
         </is>
       </c>
       <c r="E363" s="8" t="inlineStr">
@@ -28565,7 +28565,7 @@
       </c>
       <c r="D364" s="6" t="inlineStr">
         <is>
-          <t>WEB-05</t>
+          <t>ISMS-WEB-05</t>
         </is>
       </c>
       <c r="E364" s="8" t="inlineStr">
@@ -28632,7 +28632,7 @@
       </c>
       <c r="D365" s="6" t="inlineStr">
         <is>
-          <t>WEB-06</t>
+          <t>ISMS-WEB-06</t>
         </is>
       </c>
       <c r="E365" s="8" t="inlineStr">
@@ -28697,7 +28697,7 @@
       </c>
       <c r="D366" s="6" t="inlineStr">
         <is>
-          <t>WEB-10</t>
+          <t>ISMS-WEB-10</t>
         </is>
       </c>
       <c r="E366" s="8" t="inlineStr">
@@ -28766,7 +28766,7 @@
       </c>
       <c r="D367" s="6" t="inlineStr">
         <is>
-          <t>WEB-14</t>
+          <t>ISMS-WEB-14</t>
         </is>
       </c>
       <c r="E367" s="8" t="inlineStr">
@@ -28825,7 +28825,7 @@
       </c>
       <c r="D368" s="6" t="inlineStr">
         <is>
-          <t>WEB-16</t>
+          <t>ISMS-WEB-16</t>
         </is>
       </c>
       <c r="E368" s="8" t="inlineStr">
@@ -28882,7 +28882,7 @@
       </c>
       <c r="D369" s="6" t="inlineStr">
         <is>
-          <t>WEB-17</t>
+          <t>ISMS-WEB-17</t>
         </is>
       </c>
       <c r="E369" s="8" t="inlineStr">
@@ -28953,7 +28953,7 @@
       </c>
       <c r="D370" s="6" t="inlineStr">
         <is>
-          <t>WEB-18</t>
+          <t>ISMS-WEB-18</t>
         </is>
       </c>
       <c r="E370" s="8" t="inlineStr">
@@ -29028,7 +29028,7 @@
       </c>
       <c r="D371" s="6" t="inlineStr">
         <is>
-          <t>WEB-19</t>
+          <t>ISMS-WEB-19</t>
         </is>
       </c>
       <c r="E371" s="8" t="inlineStr">
@@ -29101,7 +29101,7 @@
       </c>
       <c r="D372" s="6" t="inlineStr">
         <is>
-          <t>WEB-20</t>
+          <t>ISMS-WEB-20</t>
         </is>
       </c>
       <c r="E372" s="8" t="inlineStr">
@@ -29200,7 +29200,7 @@
       </c>
       <c r="D373" s="6" t="inlineStr">
         <is>
-          <t>WEB-21</t>
+          <t>ISMS-WEB-21</t>
         </is>
       </c>
       <c r="E373" s="8" t="inlineStr">
@@ -29285,7 +29285,7 @@
       </c>
       <c r="D374" s="6" t="inlineStr">
         <is>
-          <t>WEB-22</t>
+          <t>ISMS-WEB-22</t>
         </is>
       </c>
       <c r="E374" s="8" t="inlineStr">
@@ -29372,7 +29372,7 @@
       </c>
       <c r="D375" s="6" t="inlineStr">
         <is>
-          <t>WEB-24</t>
+          <t>ISMS-WEB-24</t>
         </is>
       </c>
       <c r="E375" s="8" t="inlineStr">
@@ -29460,7 +29460,7 @@
       </c>
       <c r="D376" s="6" t="inlineStr">
         <is>
-          <t>WEB-25</t>
+          <t>ISMS-WEB-25</t>
         </is>
       </c>
       <c r="E376" s="8" t="inlineStr">
@@ -29524,7 +29524,7 @@
       </c>
       <c r="D377" s="6" t="inlineStr">
         <is>
-          <t>WEB-26</t>
+          <t>ISMS-WEB-26</t>
         </is>
       </c>
       <c r="E377" s="8" t="inlineStr">
@@ -29600,7 +29600,7 @@
       </c>
       <c r="D379" s="6" t="inlineStr">
         <is>
-          <t>CLD-Tomcat-01 / WEB-01</t>
+          <t>CSAP-Tomcat-01 / ISMS-WEB-01</t>
         </is>
       </c>
       <c r="E379" s="8" t="inlineStr">
@@ -29694,7 +29694,7 @@
       </c>
       <c r="D380" s="6" t="inlineStr">
         <is>
-          <t>CLD-Tomcat-02 / WEB-02</t>
+          <t>CSAP-Tomcat-02 / ISMS-WEB-02</t>
         </is>
       </c>
       <c r="E380" s="8" t="inlineStr">
@@ -29777,7 +29777,7 @@
       </c>
       <c r="D381" s="6" t="inlineStr">
         <is>
-          <t>CLD-Tomcat-03 / WEB-03</t>
+          <t>CSAP-Tomcat-03 / ISMS-WEB-03</t>
         </is>
       </c>
       <c r="E381" s="8" t="inlineStr">
@@ -29850,7 +29850,7 @@
       </c>
       <c r="D382" s="6" t="inlineStr">
         <is>
-          <t>CLD-Tomcat-06 / WEB-04</t>
+          <t>CSAP-Tomcat-06 / ISMS-WEB-04</t>
         </is>
       </c>
       <c r="E382" s="8" t="inlineStr">
@@ -29927,7 +29927,7 @@
       </c>
       <c r="D383" s="6" t="inlineStr">
         <is>
-          <t>CLD-Tomcat-07 / WEB-22</t>
+          <t>CSAP-Tomcat-07 / ISMS-WEB-22</t>
         </is>
       </c>
       <c r="E383" s="8" t="inlineStr">
@@ -30014,7 +30014,7 @@
       </c>
       <c r="D384" s="6" t="inlineStr">
         <is>
-          <t>CLD-Tomcat-04</t>
+          <t>CSAP-Tomcat-04</t>
         </is>
       </c>
       <c r="E384" s="8" t="inlineStr">
@@ -30068,7 +30068,7 @@
       </c>
       <c r="D385" s="6" t="inlineStr">
         <is>
-          <t>CLD-Tomcat-05</t>
+          <t>CSAP-Tomcat-05</t>
         </is>
       </c>
       <c r="E385" s="8" t="inlineStr">
@@ -30126,7 +30126,7 @@
       </c>
       <c r="D386" s="6" t="inlineStr">
         <is>
-          <t>CLD-Tomcat-08</t>
+          <t>CSAP-Tomcat-08</t>
         </is>
       </c>
       <c r="E386" s="8" t="inlineStr">
@@ -30179,7 +30179,7 @@
       </c>
       <c r="D387" s="6" t="inlineStr">
         <is>
-          <t>CLD-Tomcat-09</t>
+          <t>CSAP-Tomcat-09</t>
         </is>
       </c>
       <c r="E387" s="8" t="inlineStr">
@@ -30231,7 +30231,7 @@
       </c>
       <c r="D388" s="6" t="inlineStr">
         <is>
-          <t>WEB-05</t>
+          <t>ISMS-WEB-05</t>
         </is>
       </c>
       <c r="E388" s="8" t="inlineStr">
@@ -30296,7 +30296,7 @@
       </c>
       <c r="D389" s="6" t="inlineStr">
         <is>
-          <t>WEB-06</t>
+          <t>ISMS-WEB-06</t>
         </is>
       </c>
       <c r="E389" s="8" t="inlineStr">
@@ -30377,7 +30377,7 @@
       </c>
       <c r="D390" s="6" t="inlineStr">
         <is>
-          <t>WEB-07</t>
+          <t>ISMS-WEB-07</t>
         </is>
       </c>
       <c r="E390" s="8" t="inlineStr">
@@ -30440,7 +30440,7 @@
       </c>
       <c r="D391" s="6" t="inlineStr">
         <is>
-          <t>WEB-08</t>
+          <t>ISMS-WEB-08</t>
         </is>
       </c>
       <c r="E391" s="8" t="inlineStr">
@@ -30527,7 +30527,7 @@
       </c>
       <c r="D392" s="6" t="inlineStr">
         <is>
-          <t>WEB-09</t>
+          <t>ISMS-WEB-09</t>
         </is>
       </c>
       <c r="E392" s="8" t="inlineStr">
@@ -30611,7 +30611,7 @@
       </c>
       <c r="D393" s="6" t="inlineStr">
         <is>
-          <t>WEB-10</t>
+          <t>ISMS-WEB-10</t>
         </is>
       </c>
       <c r="E393" s="8" t="inlineStr">
@@ -30676,7 +30676,7 @@
       </c>
       <c r="D394" s="6" t="inlineStr">
         <is>
-          <t>WEB-11</t>
+          <t>ISMS-WEB-11</t>
         </is>
       </c>
       <c r="E394" s="8" t="inlineStr">
@@ -30739,7 +30739,7 @@
       </c>
       <c r="D395" s="6" t="inlineStr">
         <is>
-          <t>WEB-12</t>
+          <t>ISMS-WEB-12</t>
         </is>
       </c>
       <c r="E395" s="8" t="inlineStr">
@@ -30804,7 +30804,7 @@
       </c>
       <c r="D396" s="6" t="inlineStr">
         <is>
-          <t>WEB-13</t>
+          <t>ISMS-WEB-13</t>
         </is>
       </c>
       <c r="E396" s="8" t="inlineStr">
@@ -30891,7 +30891,7 @@
       </c>
       <c r="D397" s="6" t="inlineStr">
         <is>
-          <t>WEB-14</t>
+          <t>ISMS-WEB-14</t>
         </is>
       </c>
       <c r="E397" s="8" t="inlineStr">
@@ -30952,7 +30952,7 @@
       </c>
       <c r="D398" s="6" t="inlineStr">
         <is>
-          <t>WEB-15</t>
+          <t>ISMS-WEB-15</t>
         </is>
       </c>
       <c r="E398" s="8" t="inlineStr">
@@ -31019,7 +31019,7 @@
       </c>
       <c r="D399" s="6" t="inlineStr">
         <is>
-          <t>WEB-16</t>
+          <t>ISMS-WEB-16</t>
         </is>
       </c>
       <c r="E399" s="8" t="inlineStr">
@@ -31098,7 +31098,7 @@
       </c>
       <c r="D400" s="6" t="inlineStr">
         <is>
-          <t>WEB-17</t>
+          <t>ISMS-WEB-17</t>
         </is>
       </c>
       <c r="E400" s="8" t="inlineStr">
@@ -31163,7 +31163,7 @@
       </c>
       <c r="D401" s="6" t="inlineStr">
         <is>
-          <t>WEB-19</t>
+          <t>ISMS-WEB-19</t>
         </is>
       </c>
       <c r="E401" s="8" t="inlineStr">
@@ -31246,7 +31246,7 @@
       </c>
       <c r="D402" s="6" t="inlineStr">
         <is>
-          <t>WEB-23</t>
+          <t>ISMS-WEB-23</t>
         </is>
       </c>
       <c r="E402" s="8" t="inlineStr">
@@ -31321,7 +31321,7 @@
       </c>
       <c r="D403" s="6" t="inlineStr">
         <is>
-          <t>WEB-24</t>
+          <t>ISMS-WEB-24</t>
         </is>
       </c>
       <c r="E403" s="8" t="inlineStr">
@@ -31401,7 +31401,7 @@
       </c>
       <c r="D404" s="6" t="inlineStr">
         <is>
-          <t>WEB-25</t>
+          <t>ISMS-WEB-25</t>
         </is>
       </c>
       <c r="E404" s="8" t="inlineStr">
@@ -31467,7 +31467,7 @@
       </c>
       <c r="D405" s="6" t="inlineStr">
         <is>
-          <t>WEB-26</t>
+          <t>ISMS-WEB-26</t>
         </is>
       </c>
       <c r="E405" s="8" t="inlineStr">
@@ -31547,7 +31547,7 @@
       </c>
       <c r="D407" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-01</t>
+          <t>CSAP-Docker-01</t>
         </is>
       </c>
       <c r="E407" s="8" t="inlineStr">
@@ -31602,7 +31602,7 @@
       </c>
       <c r="D408" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-02</t>
+          <t>CSAP-Docker-02</t>
         </is>
       </c>
       <c r="E408" s="8" t="inlineStr">
@@ -31659,7 +31659,7 @@
       </c>
       <c r="D409" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-03</t>
+          <t>CSAP-Docker-03</t>
         </is>
       </c>
       <c r="E409" s="8" t="inlineStr">
@@ -31714,7 +31714,7 @@
       </c>
       <c r="D410" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-04</t>
+          <t>CSAP-Docker-04</t>
         </is>
       </c>
       <c r="E410" s="8" t="inlineStr">
@@ -31769,7 +31769,7 @@
       </c>
       <c r="D411" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-05</t>
+          <t>CSAP-Docker-05</t>
         </is>
       </c>
       <c r="E411" s="8" t="inlineStr">
@@ -31824,7 +31824,7 @@
       </c>
       <c r="D412" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-06</t>
+          <t>CSAP-Docker-06</t>
         </is>
       </c>
       <c r="E412" s="8" t="inlineStr">
@@ -31879,7 +31879,7 @@
       </c>
       <c r="D413" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-07</t>
+          <t>CSAP-Docker-07</t>
         </is>
       </c>
       <c r="E413" s="8" t="inlineStr">
@@ -31934,7 +31934,7 @@
       </c>
       <c r="D414" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-08</t>
+          <t>CSAP-Docker-08</t>
         </is>
       </c>
       <c r="E414" s="8" t="inlineStr">
@@ -31991,7 +31991,7 @@
       </c>
       <c r="D415" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-09</t>
+          <t>CSAP-Docker-09</t>
         </is>
       </c>
       <c r="E415" s="8" t="inlineStr">
@@ -32049,7 +32049,7 @@
       </c>
       <c r="D416" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-10</t>
+          <t>CSAP-Docker-10</t>
         </is>
       </c>
       <c r="E416" s="8" t="inlineStr">
@@ -32114,7 +32114,7 @@
       </c>
       <c r="D417" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-11</t>
+          <t>CSAP-Docker-11</t>
         </is>
       </c>
       <c r="E417" s="8" t="inlineStr">
@@ -32166,7 +32166,7 @@
       </c>
       <c r="D418" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-12</t>
+          <t>CSAP-Docker-12</t>
         </is>
       </c>
       <c r="E418" s="8" t="inlineStr">
@@ -32221,7 +32221,7 @@
       </c>
       <c r="D419" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-13</t>
+          <t>CSAP-Docker-13</t>
         </is>
       </c>
       <c r="E419" s="8" t="inlineStr">
@@ -32273,7 +32273,7 @@
       </c>
       <c r="D420" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-14</t>
+          <t>CSAP-Docker-14</t>
         </is>
       </c>
       <c r="E420" s="8" t="inlineStr">
@@ -32326,7 +32326,7 @@
       </c>
       <c r="D421" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-15</t>
+          <t>CSAP-Docker-15</t>
         </is>
       </c>
       <c r="E421" s="8" t="inlineStr">
@@ -32379,7 +32379,7 @@
       </c>
       <c r="D422" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-16</t>
+          <t>CSAP-Docker-16</t>
         </is>
       </c>
       <c r="E422" s="8" t="inlineStr">
@@ -32431,7 +32431,7 @@
       </c>
       <c r="D423" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-17</t>
+          <t>CSAP-Docker-17</t>
         </is>
       </c>
       <c r="E423" s="8" t="inlineStr">
@@ -32482,7 +32482,7 @@
       </c>
       <c r="D424" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-18</t>
+          <t>CSAP-Docker-18</t>
         </is>
       </c>
       <c r="E424" s="8" t="inlineStr">
@@ -32529,7 +32529,7 @@
       </c>
       <c r="D425" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-19</t>
+          <t>CSAP-Docker-19</t>
         </is>
       </c>
       <c r="E425" s="8" t="inlineStr">
@@ -32581,7 +32581,7 @@
       </c>
       <c r="D426" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-20</t>
+          <t>CSAP-Docker-20</t>
         </is>
       </c>
       <c r="E426" s="8" t="inlineStr">
@@ -32632,7 +32632,7 @@
       </c>
       <c r="D427" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-21</t>
+          <t>CSAP-Docker-21</t>
         </is>
       </c>
       <c r="E427" s="8" t="inlineStr">
@@ -32683,7 +32683,7 @@
       </c>
       <c r="D428" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-22</t>
+          <t>CSAP-Docker-22</t>
         </is>
       </c>
       <c r="E428" s="8" t="inlineStr">
@@ -32734,7 +32734,7 @@
       </c>
       <c r="D429" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-23</t>
+          <t>CSAP-Docker-23</t>
         </is>
       </c>
       <c r="E429" s="8" t="inlineStr">
@@ -32787,7 +32787,7 @@
       </c>
       <c r="D430" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-24</t>
+          <t>CSAP-Docker-24</t>
         </is>
       </c>
       <c r="E430" s="8" t="inlineStr">
@@ -32840,7 +32840,7 @@
       </c>
       <c r="D431" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-25</t>
+          <t>CSAP-Docker-25</t>
         </is>
       </c>
       <c r="E431" s="8" t="inlineStr">
@@ -32892,7 +32892,7 @@
       </c>
       <c r="D432" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-26</t>
+          <t>CSAP-Docker-26</t>
         </is>
       </c>
       <c r="E432" s="8" t="inlineStr">
@@ -32945,7 +32945,7 @@
       </c>
       <c r="D433" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-27</t>
+          <t>CSAP-Docker-27</t>
         </is>
       </c>
       <c r="E433" s="8" t="inlineStr">
@@ -33000,7 +33000,7 @@
       </c>
       <c r="D434" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-28</t>
+          <t>CSAP-Docker-28</t>
         </is>
       </c>
       <c r="E434" s="8" t="inlineStr">
@@ -33050,7 +33050,7 @@
       </c>
       <c r="D435" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-29</t>
+          <t>CSAP-Docker-29</t>
         </is>
       </c>
       <c r="E435" s="8" t="inlineStr">
@@ -33100,7 +33100,7 @@
       </c>
       <c r="D436" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-30</t>
+          <t>CSAP-Docker-30</t>
         </is>
       </c>
       <c r="E436" s="8" t="inlineStr">
@@ -33151,7 +33151,7 @@
       </c>
       <c r="D437" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-31</t>
+          <t>CSAP-Docker-31</t>
         </is>
       </c>
       <c r="E437" s="8" t="inlineStr">
@@ -33211,7 +33211,7 @@
       </c>
       <c r="D438" s="6" t="inlineStr">
         <is>
-          <t>CLD-Docker-32</t>
+          <t>CSAP-Docker-32</t>
         </is>
       </c>
       <c r="E438" s="8" t="inlineStr">
@@ -33275,7 +33275,7 @@
       </c>
       <c r="D440" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sMaster-01</t>
+          <t>CSAP-K8sMaster-01</t>
         </is>
       </c>
       <c r="E440" s="8" t="inlineStr">
@@ -33328,7 +33328,7 @@
       </c>
       <c r="D441" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sMaster-02</t>
+          <t>CSAP-K8sMaster-02</t>
         </is>
       </c>
       <c r="E441" s="8" t="inlineStr">
@@ -33379,7 +33379,7 @@
       </c>
       <c r="D442" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sMaster-03</t>
+          <t>CSAP-K8sMaster-03</t>
         </is>
       </c>
       <c r="E442" s="8" t="inlineStr">
@@ -33435,7 +33435,7 @@
       </c>
       <c r="D443" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sMaster-04</t>
+          <t>CSAP-K8sMaster-04</t>
         </is>
       </c>
       <c r="E443" s="8" t="inlineStr">
@@ -33500,7 +33500,7 @@
       </c>
       <c r="D444" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sMaster-05</t>
+          <t>CSAP-K8sMaster-05</t>
         </is>
       </c>
       <c r="E444" s="8" t="inlineStr">
@@ -33564,7 +33564,7 @@
       </c>
       <c r="D445" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sMaster-06</t>
+          <t>CSAP-K8sMaster-06</t>
         </is>
       </c>
       <c r="E445" s="8" t="inlineStr">
@@ -33650,7 +33650,7 @@
       </c>
       <c r="D446" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sMaster-07</t>
+          <t>CSAP-K8sMaster-07</t>
         </is>
       </c>
       <c r="E446" s="8" t="inlineStr">
@@ -33705,7 +33705,7 @@
       </c>
       <c r="D447" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sMaster-08</t>
+          <t>CSAP-K8sMaster-08</t>
         </is>
       </c>
       <c r="E447" s="8" t="inlineStr">
@@ -33769,7 +33769,7 @@
       </c>
       <c r="D448" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sMaster-09</t>
+          <t>CSAP-K8sMaster-09</t>
         </is>
       </c>
       <c r="E448" s="8" t="inlineStr">
@@ -33831,7 +33831,7 @@
       </c>
       <c r="D449" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sMaster-10</t>
+          <t>CSAP-K8sMaster-10</t>
         </is>
       </c>
       <c r="E449" s="8" t="inlineStr">
@@ -33893,7 +33893,7 @@
       </c>
       <c r="D450" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sMaster-11</t>
+          <t>CSAP-K8sMaster-11</t>
         </is>
       </c>
       <c r="E450" s="8" t="inlineStr">
@@ -33979,7 +33979,7 @@
       </c>
       <c r="D451" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sMaster-12</t>
+          <t>CSAP-K8sMaster-12</t>
         </is>
       </c>
       <c r="E451" s="8" t="inlineStr">
@@ -34050,7 +34050,7 @@
       </c>
       <c r="D452" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sMaster-13</t>
+          <t>CSAP-K8sMaster-13</t>
         </is>
       </c>
       <c r="E452" s="8" t="inlineStr">
@@ -34105,7 +34105,7 @@
       </c>
       <c r="D453" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sMaster-14</t>
+          <t>CSAP-K8sMaster-14</t>
         </is>
       </c>
       <c r="E453" s="8" t="inlineStr">
@@ -34181,7 +34181,7 @@
       </c>
       <c r="D454" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sMaster-15</t>
+          <t>CSAP-K8sMaster-15</t>
         </is>
       </c>
       <c r="E454" s="8" t="inlineStr">
@@ -34242,7 +34242,7 @@
       </c>
       <c r="D455" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sMaster-16</t>
+          <t>CSAP-K8sMaster-16</t>
         </is>
       </c>
       <c r="E455" s="8" t="inlineStr">
@@ -34295,7 +34295,7 @@
       </c>
       <c r="D456" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sMaster-17</t>
+          <t>CSAP-K8sMaster-17</t>
         </is>
       </c>
       <c r="E456" s="8" t="inlineStr">
@@ -34366,7 +34366,7 @@
       </c>
       <c r="D458" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sWorker-01</t>
+          <t>CSAP-K8sWorker-01</t>
         </is>
       </c>
       <c r="E458" s="8" t="inlineStr">
@@ -34435,7 +34435,7 @@
       </c>
       <c r="D459" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sWorker-02</t>
+          <t>CSAP-K8sWorker-02</t>
         </is>
       </c>
       <c r="E459" s="8" t="inlineStr">
@@ -34497,7 +34497,7 @@
       </c>
       <c r="D460" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sWorker-03</t>
+          <t>CSAP-K8sWorker-03</t>
         </is>
       </c>
       <c r="E460" s="8" t="inlineStr">
@@ -34584,7 +34584,7 @@
       </c>
       <c r="D461" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sWorker-04</t>
+          <t>CSAP-K8sWorker-04</t>
         </is>
       </c>
       <c r="E461" s="8" t="inlineStr">
@@ -34646,7 +34646,7 @@
       </c>
       <c r="D462" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sWorker-05</t>
+          <t>CSAP-K8sWorker-05</t>
         </is>
       </c>
       <c r="E462" s="8" t="inlineStr">
@@ -34708,7 +34708,7 @@
       </c>
       <c r="D463" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sWorker-06</t>
+          <t>CSAP-K8sWorker-06</t>
         </is>
       </c>
       <c r="E463" s="8" t="inlineStr">
@@ -34762,7 +34762,7 @@
       </c>
       <c r="D464" s="6" t="inlineStr">
         <is>
-          <t>CLD-K8sWorker-07</t>
+          <t>CSAP-K8sWorker-07</t>
         </is>
       </c>
       <c r="E464" s="8" t="inlineStr">
@@ -34827,7 +34827,7 @@
       </c>
       <c r="D466" s="6" t="inlineStr">
         <is>
-          <t>CLD-PHP-01</t>
+          <t>CSAP-PHP-01</t>
         </is>
       </c>
       <c r="E466" s="8" t="inlineStr">
@@ -34877,7 +34877,7 @@
       </c>
       <c r="D467" s="6" t="inlineStr">
         <is>
-          <t>CLD-PHP-02</t>
+          <t>CSAP-PHP-02</t>
         </is>
       </c>
       <c r="E467" s="8" t="inlineStr">
@@ -34926,7 +34926,7 @@
       </c>
       <c r="D468" s="6" t="inlineStr">
         <is>
-          <t>CLD-PHP-03</t>
+          <t>CSAP-PHP-03</t>
         </is>
       </c>
       <c r="E468" s="8" t="inlineStr">
@@ -34975,7 +34975,7 @@
       </c>
       <c r="D469" s="6" t="inlineStr">
         <is>
-          <t>CLD-PHP-04</t>
+          <t>CSAP-PHP-04</t>
         </is>
       </c>
       <c r="E469" s="8" t="inlineStr">
@@ -35034,7 +35034,7 @@
       </c>
       <c r="D470" s="6" t="inlineStr">
         <is>
-          <t>CLD-PHP-05</t>
+          <t>CSAP-PHP-05</t>
         </is>
       </c>
       <c r="E470" s="8" t="inlineStr">
@@ -35086,7 +35086,7 @@
       </c>
       <c r="D471" s="6" t="inlineStr">
         <is>
-          <t>CLD-PHP-06</t>
+          <t>CSAP-PHP-06</t>
         </is>
       </c>
       <c r="E471" s="8" t="inlineStr">
@@ -35151,7 +35151,7 @@
       </c>
       <c r="D473" s="6" t="inlineStr">
         <is>
-          <t>CLD-NodeJS-01</t>
+          <t>CSAP-NodeJS-01</t>
         </is>
       </c>
       <c r="E473" s="8" t="inlineStr">
@@ -35214,7 +35214,7 @@
       </c>
       <c r="D474" s="6" t="inlineStr">
         <is>
-          <t>CLD-NodeJS-02</t>
+          <t>CSAP-NodeJS-02</t>
         </is>
       </c>
       <c r="E474" s="8" t="inlineStr">
@@ -35265,7 +35265,7 @@
       </c>
       <c r="D475" s="6" t="inlineStr">
         <is>
-          <t>CLD-NodeJS-03</t>
+          <t>CSAP-NodeJS-03</t>
         </is>
       </c>
       <c r="E475" s="8" t="inlineStr">
@@ -35323,7 +35323,7 @@
       </c>
       <c r="D476" s="6" t="inlineStr">
         <is>
-          <t>CLD-NodeJS-04</t>
+          <t>CSAP-NodeJS-04</t>
         </is>
       </c>
       <c r="E476" s="8" t="inlineStr">
@@ -35384,7 +35384,7 @@
       </c>
       <c r="D477" s="6" t="inlineStr">
         <is>
-          <t>CLD-NodeJS-05</t>
+          <t>CSAP-NodeJS-05</t>
         </is>
       </c>
       <c r="E477" s="8" t="inlineStr">
@@ -35461,7 +35461,7 @@
       </c>
       <c r="D478" s="6" t="inlineStr">
         <is>
-          <t>CLD-NodeJS-06</t>
+          <t>CSAP-NodeJS-06</t>
         </is>
       </c>
       <c r="E478" s="8" t="inlineStr">
@@ -35520,7 +35520,7 @@
       </c>
       <c r="D479" s="6" t="inlineStr">
         <is>
-          <t>CLD-NodeJS-07</t>
+          <t>CSAP-NodeJS-07</t>
         </is>
       </c>
       <c r="E479" s="8" t="inlineStr">
@@ -35598,7 +35598,7 @@
       </c>
       <c r="D481" s="6" t="inlineStr">
         <is>
-          <t>CLD-Hadoop-01</t>
+          <t>CSAP-Hadoop-01</t>
         </is>
       </c>
       <c r="E481" s="8" t="inlineStr">
@@ -35671,7 +35671,7 @@
       </c>
       <c r="D482" s="6" t="inlineStr">
         <is>
-          <t>CLD-Hadoop-02</t>
+          <t>CSAP-Hadoop-02</t>
         </is>
       </c>
       <c r="E482" s="8" t="inlineStr">
@@ -35726,7 +35726,7 @@
       </c>
       <c r="D483" s="6" t="inlineStr">
         <is>
-          <t>CLD-Hadoop-03</t>
+          <t>CSAP-Hadoop-03</t>
         </is>
       </c>
       <c r="E483" s="8" t="inlineStr">
@@ -35775,7 +35775,7 @@
       </c>
       <c r="D484" s="6" t="inlineStr">
         <is>
-          <t>CLD-Hadoop-04</t>
+          <t>CSAP-Hadoop-04</t>
         </is>
       </c>
       <c r="E484" s="8" t="inlineStr">
@@ -35828,7 +35828,7 @@
       </c>
       <c r="D485" s="6" t="inlineStr">
         <is>
-          <t>CLD-Hadoop-05</t>
+          <t>CSAP-Hadoop-05</t>
         </is>
       </c>
       <c r="E485" s="8" t="inlineStr">
@@ -35880,7 +35880,7 @@
       </c>
       <c r="D486" s="6" t="inlineStr">
         <is>
-          <t>CLD-Hadoop-06</t>
+          <t>CSAP-Hadoop-06</t>
         </is>
       </c>
       <c r="E486" s="8" t="inlineStr">
@@ -35930,7 +35930,7 @@
       </c>
       <c r="D487" s="6" t="inlineStr">
         <is>
-          <t>CLD-Hadoop-07</t>
+          <t>CSAP-Hadoop-07</t>
         </is>
       </c>
       <c r="E487" s="8" t="inlineStr">
@@ -35988,7 +35988,7 @@
       </c>
       <c r="D488" s="6" t="inlineStr">
         <is>
-          <t>CLD-Hadoop-08</t>
+          <t>CSAP-Hadoop-08</t>
         </is>
       </c>
       <c r="E488" s="8" t="inlineStr">
@@ -36043,7 +36043,7 @@
       </c>
       <c r="D489" s="6" t="inlineStr">
         <is>
-          <t>CLD-Hadoop-09</t>
+          <t>CSAP-Hadoop-09</t>
         </is>
       </c>
       <c r="E489" s="8" t="inlineStr">
@@ -36110,7 +36110,7 @@
       </c>
       <c r="D491" s="6" t="inlineStr">
         <is>
-          <t>CLD-Ceph-01</t>
+          <t>CSAP-Ceph-01</t>
         </is>
       </c>
       <c r="E491" s="8" t="inlineStr">
@@ -36165,7 +36165,7 @@
       </c>
       <c r="D492" s="6" t="inlineStr">
         <is>
-          <t>CLD-Ceph-02</t>
+          <t>CSAP-Ceph-02</t>
         </is>
       </c>
       <c r="E492" s="8" t="inlineStr">
@@ -36221,7 +36221,7 @@
       </c>
       <c r="D493" s="6" t="inlineStr">
         <is>
-          <t>CLD-Ceph-03</t>
+          <t>CSAP-Ceph-03</t>
         </is>
       </c>
       <c r="E493" s="8" t="inlineStr">
@@ -36271,7 +36271,7 @@
       </c>
       <c r="D494" s="6" t="inlineStr">
         <is>
-          <t>CLD-Ceph-04</t>
+          <t>CSAP-Ceph-04</t>
         </is>
       </c>
       <c r="E494" s="8" t="inlineStr">
@@ -36319,7 +36319,7 @@
       </c>
       <c r="D495" s="6" t="inlineStr">
         <is>
-          <t>CLD-Ceph-05</t>
+          <t>CSAP-Ceph-05</t>
         </is>
       </c>
       <c r="E495" s="8" t="inlineStr">
@@ -36375,7 +36375,7 @@
       </c>
       <c r="D496" s="6" t="inlineStr">
         <is>
-          <t>CLD-Ceph-06</t>
+          <t>CSAP-Ceph-06</t>
         </is>
       </c>
       <c r="E496" s="8" t="inlineStr">
@@ -36419,7 +36419,7 @@
       </c>
       <c r="D497" s="6" t="inlineStr">
         <is>
-          <t>CLD-Ceph-07</t>
+          <t>CSAP-Ceph-07</t>
         </is>
       </c>
       <c r="E497" s="8" t="inlineStr">

</xml_diff>